<commit_message>
added ghg for building material
</commit_message>
<xml_diff>
--- a/data_input/MI_Buildings_Oorschot2023MetabolicMPG.xlsx
+++ b/data_input/MI_Buildings_Oorschot2023MetabolicMPG.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Mira/Documents/IE/REAL UTOPIAN HOUSING/Post-GrowthHousingScenarios/Code/housing-footprints/data_input/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A218D8BB-A247-7A4C-BF3E-A11BBFAA1AFC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C46774F7-8DDB-B04E-886E-6F75251CEAC4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="27820" yWindow="500" windowWidth="21680" windowHeight="19900" xr2:uid="{CAA754D3-AC81-B346-A139-F28AD287D6E3}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="25600" windowHeight="15500" xr2:uid="{CAA754D3-AC81-B346-A139-F28AD287D6E3}"/>
   </bookViews>
   <sheets>
     <sheet name="Building_MI" sheetId="6" r:id="rId1"/>
@@ -63,7 +63,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="635" uniqueCount="165">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="641" uniqueCount="166">
   <si>
     <t>Building type</t>
   </si>
@@ -559,6 +559,9 @@
   <si>
     <t>pre 1945</t>
   </si>
+  <si>
+    <t>semi-detached (2-1 kap) / corner (hoek)</t>
+  </si>
 </sst>
 </file>
 
@@ -875,7 +878,7 @@
             <c:multiLvlStrRef>
               <c:f>Building_MI!$A$6:$B$25</c:f>
               <c:multiLvlStrCache>
-                <c:ptCount val="15"/>
+                <c:ptCount val="20"/>
                 <c:lvl>
                   <c:pt idx="0">
                     <c:v>pre 1945</c:v>
@@ -920,6 +923,21 @@
                     <c:v>2000-2018</c:v>
                   </c:pt>
                   <c:pt idx="14">
+                    <c:v>2018-2050</c:v>
+                  </c:pt>
+                  <c:pt idx="15">
+                    <c:v>pre 1945</c:v>
+                  </c:pt>
+                  <c:pt idx="16">
+                    <c:v>1945-1970</c:v>
+                  </c:pt>
+                  <c:pt idx="17">
+                    <c:v>1970-2000</c:v>
+                  </c:pt>
+                  <c:pt idx="18">
+                    <c:v>2000-2018</c:v>
+                  </c:pt>
+                  <c:pt idx="19">
                     <c:v>2018-2050</c:v>
                   </c:pt>
                 </c:lvl>
@@ -928,9 +946,12 @@
                     <c:v>detached (vrijstaand)</c:v>
                   </c:pt>
                   <c:pt idx="5">
+                    <c:v>semi-detached (2-1 kap) / corner (hoek)</c:v>
+                  </c:pt>
+                  <c:pt idx="10">
                     <c:v>row house (tussenwoning)</c:v>
                   </c:pt>
-                  <c:pt idx="10">
+                  <c:pt idx="15">
                     <c:v>multiple fam (meergezins)</c:v>
                   </c:pt>
                 </c:lvl>
@@ -959,33 +980,48 @@
                   <c:v>1.8059701492537312</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.3463036371951419</c:v>
+                  <c:v>0.18886813098591554</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0.42903842399299175</c:v>
+                  <c:v>0.28178136220657279</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0.3567510263533375</c:v>
+                  <c:v>0.25258702535211269</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>0.35675102635333744</c:v>
+                  <c:v>0.25258702535211269</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>1.3014110606388347</c:v>
+                  <c:v>1.8059701492537312</c:v>
                 </c:pt>
                 <c:pt idx="10">
+                  <c:v>0.37854946376811599</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>0.45919950893719808</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>0.37808582173913052</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>0.37808582173913047</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>1.1980676328502415</c:v>
+                </c:pt>
+                <c:pt idx="15">
                   <c:v>0.20221829725790513</c:v>
                 </c:pt>
-                <c:pt idx="11">
+                <c:pt idx="16">
                   <c:v>0.30659409121376718</c:v>
                 </c:pt>
-                <c:pt idx="12">
+                <c:pt idx="17">
                   <c:v>0.78220971588438193</c:v>
                 </c:pt>
-                <c:pt idx="13">
+                <c:pt idx="18">
                   <c:v>0.78220971588438182</c:v>
                 </c:pt>
-                <c:pt idx="14">
+                <c:pt idx="19">
                   <c:v>1.5489130434782608</c:v>
                 </c:pt>
               </c:numCache>
@@ -1025,7 +1061,7 @@
             <c:multiLvlStrRef>
               <c:f>Building_MI!$A$6:$B$25</c:f>
               <c:multiLvlStrCache>
-                <c:ptCount val="15"/>
+                <c:ptCount val="20"/>
                 <c:lvl>
                   <c:pt idx="0">
                     <c:v>pre 1945</c:v>
@@ -1070,6 +1106,21 @@
                     <c:v>2000-2018</c:v>
                   </c:pt>
                   <c:pt idx="14">
+                    <c:v>2018-2050</c:v>
+                  </c:pt>
+                  <c:pt idx="15">
+                    <c:v>pre 1945</c:v>
+                  </c:pt>
+                  <c:pt idx="16">
+                    <c:v>1945-1970</c:v>
+                  </c:pt>
+                  <c:pt idx="17">
+                    <c:v>1970-2000</c:v>
+                  </c:pt>
+                  <c:pt idx="18">
+                    <c:v>2000-2018</c:v>
+                  </c:pt>
+                  <c:pt idx="19">
                     <c:v>2018-2050</c:v>
                   </c:pt>
                 </c:lvl>
@@ -1078,9 +1129,12 @@
                     <c:v>detached (vrijstaand)</c:v>
                   </c:pt>
                   <c:pt idx="5">
+                    <c:v>semi-detached (2-1 kap) / corner (hoek)</c:v>
+                  </c:pt>
+                  <c:pt idx="10">
                     <c:v>row house (tussenwoning)</c:v>
                   </c:pt>
-                  <c:pt idx="10">
+                  <c:pt idx="15">
                     <c:v>multiple fam (meergezins)</c:v>
                   </c:pt>
                 </c:lvl>
@@ -1109,33 +1163,48 @@
                   <c:v>218.41791044776119</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>189.94763395111249</c:v>
+                  <c:v>322.16941545070426</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>170.95287055568011</c:v>
+                  <c:v>289.95247390610336</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>75.979053578518062</c:v>
+                  <c:v>128.86776618309858</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>75.979053578518062</c:v>
+                  <c:v>128.86776618309858</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>186.50297714326916</c:v>
+                  <c:v>218.41791044776119</c:v>
                 </c:pt>
                 <c:pt idx="10">
+                  <c:v>162.86606424637682</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>146.57945782125606</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>65.146425695652184</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>65.146425695652184</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>179.96618357487924</c:v>
+                </c:pt>
+                <c:pt idx="15">
                   <c:v>169.93780449011857</c:v>
                 </c:pt>
-                <c:pt idx="11">
+                <c:pt idx="16">
                   <c:v>150.70739824798255</c:v>
                 </c:pt>
-                <c:pt idx="12">
+                <c:pt idx="17">
                   <c:v>54.555367037302368</c:v>
                 </c:pt>
-                <c:pt idx="13">
+                <c:pt idx="18">
                   <c:v>54.555367037302368</c:v>
                 </c:pt>
-                <c:pt idx="14">
+                <c:pt idx="19">
                   <c:v>237.06521739130437</c:v>
                 </c:pt>
               </c:numCache>
@@ -1175,7 +1244,7 @@
             <c:multiLvlStrRef>
               <c:f>Building_MI!$A$6:$B$25</c:f>
               <c:multiLvlStrCache>
-                <c:ptCount val="15"/>
+                <c:ptCount val="20"/>
                 <c:lvl>
                   <c:pt idx="0">
                     <c:v>pre 1945</c:v>
@@ -1220,6 +1289,21 @@
                     <c:v>2000-2018</c:v>
                   </c:pt>
                   <c:pt idx="14">
+                    <c:v>2018-2050</c:v>
+                  </c:pt>
+                  <c:pt idx="15">
+                    <c:v>pre 1945</c:v>
+                  </c:pt>
+                  <c:pt idx="16">
+                    <c:v>1945-1970</c:v>
+                  </c:pt>
+                  <c:pt idx="17">
+                    <c:v>1970-2000</c:v>
+                  </c:pt>
+                  <c:pt idx="18">
+                    <c:v>2000-2018</c:v>
+                  </c:pt>
+                  <c:pt idx="19">
                     <c:v>2018-2050</c:v>
                   </c:pt>
                 </c:lvl>
@@ -1228,9 +1312,12 @@
                     <c:v>detached (vrijstaand)</c:v>
                   </c:pt>
                   <c:pt idx="5">
+                    <c:v>semi-detached (2-1 kap) / corner (hoek)</c:v>
+                  </c:pt>
+                  <c:pt idx="10">
                     <c:v>row house (tussenwoning)</c:v>
                   </c:pt>
-                  <c:pt idx="10">
+                  <c:pt idx="15">
                     <c:v>multiple fam (meergezins)</c:v>
                   </c:pt>
                 </c:lvl>
@@ -1259,33 +1346,48 @@
                   <c:v>1190.3880597014925</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>1185.8494540952004</c:v>
+                  <c:v>1388.6241446239421</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>1286.9143730009619</c:v>
+                  <c:v>1521.8742804915478</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>1353.0058488562827</c:v>
+                  <c:v>1589.920186801407</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>1353.0058488562825</c:v>
+                  <c:v>1589.920186801407</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>1582.3432165260654</c:v>
+                  <c:v>1190.3880597014925</c:v>
                 </c:pt>
                 <c:pt idx="10">
+                  <c:v>1144.3172885652173</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>1238.7900545992754</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>1304.4812254217393</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>1304.4812254217391</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>1662.6231884057972</c:v>
+                </c:pt>
+                <c:pt idx="15">
                   <c:v>1421.6139480039028</c:v>
                 </c:pt>
-                <c:pt idx="11">
+                <c:pt idx="16">
                   <c:v>1514.6210843366187</c:v>
                 </c:pt>
-                <c:pt idx="12">
+                <c:pt idx="17">
                   <c:v>1526.4957120451579</c:v>
                 </c:pt>
-                <c:pt idx="13">
+                <c:pt idx="18">
                   <c:v>1526.4957120451579</c:v>
                 </c:pt>
-                <c:pt idx="14">
+                <c:pt idx="19">
                   <c:v>1107.9076086956522</c:v>
                 </c:pt>
               </c:numCache>
@@ -1325,7 +1427,7 @@
             <c:multiLvlStrRef>
               <c:f>Building_MI!$A$6:$B$25</c:f>
               <c:multiLvlStrCache>
-                <c:ptCount val="15"/>
+                <c:ptCount val="20"/>
                 <c:lvl>
                   <c:pt idx="0">
                     <c:v>pre 1945</c:v>
@@ -1370,6 +1472,21 @@
                     <c:v>2000-2018</c:v>
                   </c:pt>
                   <c:pt idx="14">
+                    <c:v>2018-2050</c:v>
+                  </c:pt>
+                  <c:pt idx="15">
+                    <c:v>pre 1945</c:v>
+                  </c:pt>
+                  <c:pt idx="16">
+                    <c:v>1945-1970</c:v>
+                  </c:pt>
+                  <c:pt idx="17">
+                    <c:v>1970-2000</c:v>
+                  </c:pt>
+                  <c:pt idx="18">
+                    <c:v>2000-2018</c:v>
+                  </c:pt>
+                  <c:pt idx="19">
                     <c:v>2018-2050</c:v>
                   </c:pt>
                 </c:lvl>
@@ -1378,9 +1495,12 @@
                     <c:v>detached (vrijstaand)</c:v>
                   </c:pt>
                   <c:pt idx="5">
+                    <c:v>semi-detached (2-1 kap) / corner (hoek)</c:v>
+                  </c:pt>
+                  <c:pt idx="10">
                     <c:v>row house (tussenwoning)</c:v>
                   </c:pt>
-                  <c:pt idx="10">
+                  <c:pt idx="15">
                     <c:v>multiple fam (meergezins)</c:v>
                   </c:pt>
                 </c:lvl>
@@ -1421,21 +1541,36 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>0.55104621818444022</c:v>
+                  <c:v>0.10447761194029852</c:v>
                 </c:pt>
                 <c:pt idx="10">
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="11">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>0.64251207729468607</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="16">
                   <c:v>0.13764470016057295</c:v>
                 </c:pt>
-                <c:pt idx="12">
+                <c:pt idx="17">
                   <c:v>0.82586820096343772</c:v>
                 </c:pt>
-                <c:pt idx="13">
+                <c:pt idx="18">
                   <c:v>0.82586820096343772</c:v>
                 </c:pt>
-                <c:pt idx="14">
+                <c:pt idx="19">
                   <c:v>0.31521739130434784</c:v>
                 </c:pt>
               </c:numCache>
@@ -1475,7 +1610,7 @@
             <c:multiLvlStrRef>
               <c:f>Building_MI!$A$6:$B$25</c:f>
               <c:multiLvlStrCache>
-                <c:ptCount val="15"/>
+                <c:ptCount val="20"/>
                 <c:lvl>
                   <c:pt idx="0">
                     <c:v>pre 1945</c:v>
@@ -1520,6 +1655,21 @@
                     <c:v>2000-2018</c:v>
                   </c:pt>
                   <c:pt idx="14">
+                    <c:v>2018-2050</c:v>
+                  </c:pt>
+                  <c:pt idx="15">
+                    <c:v>pre 1945</c:v>
+                  </c:pt>
+                  <c:pt idx="16">
+                    <c:v>1945-1970</c:v>
+                  </c:pt>
+                  <c:pt idx="17">
+                    <c:v>1970-2000</c:v>
+                  </c:pt>
+                  <c:pt idx="18">
+                    <c:v>2000-2018</c:v>
+                  </c:pt>
+                  <c:pt idx="19">
                     <c:v>2018-2050</c:v>
                   </c:pt>
                 </c:lvl>
@@ -1528,9 +1678,12 @@
                     <c:v>detached (vrijstaand)</c:v>
                   </c:pt>
                   <c:pt idx="5">
+                    <c:v>semi-detached (2-1 kap) / corner (hoek)</c:v>
+                  </c:pt>
+                  <c:pt idx="10">
                     <c:v>row house (tussenwoning)</c:v>
                   </c:pt>
-                  <c:pt idx="10">
+                  <c:pt idx="15">
                     <c:v>multiple fam (meergezins)</c:v>
                   </c:pt>
                 </c:lvl>
@@ -1559,33 +1712,48 @@
                   <c:v>0.62686567164179097</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>1.6904236620330679E-2</c:v>
+                  <c:v>7.0422535211267607E-3</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>1.6904236620330679E-2</c:v>
+                  <c:v>7.0422535211267616E-3</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>1.6904236620330679E-2</c:v>
+                  <c:v>7.0422535211267616E-3</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>1.6904236620330679E-2</c:v>
+                  <c:v>7.0422535211267607E-3</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>0.85236426562837997</c:v>
+                  <c:v>0.62686567164179097</c:v>
                 </c:pt>
                 <c:pt idx="10">
+                  <c:v>1.8924160869565217E-2</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>1.8924160869565217E-2</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>1.8924160869565217E-2</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>1.8924160869565217E-2</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>0.89855072463768126</c:v>
+                </c:pt>
+                <c:pt idx="15">
                   <c:v>3.2032279496047429E-2</c:v>
                 </c:pt>
-                <c:pt idx="11">
+                <c:pt idx="16">
                   <c:v>3.2032279496047429E-2</c:v>
                 </c:pt>
-                <c:pt idx="12">
+                <c:pt idx="17">
                   <c:v>3.2032279496047429E-2</c:v>
                 </c:pt>
-                <c:pt idx="13">
+                <c:pt idx="18">
                   <c:v>3.2032279496047429E-2</c:v>
                 </c:pt>
-                <c:pt idx="14">
+                <c:pt idx="19">
                   <c:v>1.2880434782608696</c:v>
                 </c:pt>
               </c:numCache>
@@ -1625,7 +1793,7 @@
             <c:multiLvlStrRef>
               <c:f>Building_MI!$A$6:$B$25</c:f>
               <c:multiLvlStrCache>
-                <c:ptCount val="15"/>
+                <c:ptCount val="20"/>
                 <c:lvl>
                   <c:pt idx="0">
                     <c:v>pre 1945</c:v>
@@ -1670,6 +1838,21 @@
                     <c:v>2000-2018</c:v>
                   </c:pt>
                   <c:pt idx="14">
+                    <c:v>2018-2050</c:v>
+                  </c:pt>
+                  <c:pt idx="15">
+                    <c:v>pre 1945</c:v>
+                  </c:pt>
+                  <c:pt idx="16">
+                    <c:v>1945-1970</c:v>
+                  </c:pt>
+                  <c:pt idx="17">
+                    <c:v>1970-2000</c:v>
+                  </c:pt>
+                  <c:pt idx="18">
+                    <c:v>2000-2018</c:v>
+                  </c:pt>
+                  <c:pt idx="19">
                     <c:v>2018-2050</c:v>
                   </c:pt>
                 </c:lvl>
@@ -1678,9 +1861,12 @@
                     <c:v>detached (vrijstaand)</c:v>
                   </c:pt>
                   <c:pt idx="5">
+                    <c:v>semi-detached (2-1 kap) / corner (hoek)</c:v>
+                  </c:pt>
+                  <c:pt idx="10">
                     <c:v>row house (tussenwoning)</c:v>
                   </c:pt>
-                  <c:pt idx="10">
+                  <c:pt idx="15">
                     <c:v>multiple fam (meergezins)</c:v>
                   </c:pt>
                 </c:lvl>
@@ -1709,33 +1895,48 @@
                   <c:v>15.820895522388058</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>8.0895612976966706</c:v>
+                  <c:v>10.021588338028154</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>21.815203981267402</c:v>
+                  <c:v>46.677546563380268</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>21.815203981267402</c:v>
+                  <c:v>46.677546563380268</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>21.815203981267398</c:v>
+                  <c:v>46.677546563380261</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>13.928634364409836</c:v>
+                  <c:v>15.820895522388058</c:v>
                 </c:pt>
                 <c:pt idx="10">
+                  <c:v>7.6938449159420292</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>16.722916946376813</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>16.722916946376813</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>16.722916946376813</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>13.54106280193237</c:v>
+                </c:pt>
+                <c:pt idx="15">
                   <c:v>13.986688577099798</c:v>
                 </c:pt>
-                <c:pt idx="11">
+                <c:pt idx="16">
                   <c:v>13.822343876152829</c:v>
                 </c:pt>
-                <c:pt idx="12">
+                <c:pt idx="17">
                   <c:v>13.000620371417984</c:v>
                 </c:pt>
-                <c:pt idx="13">
+                <c:pt idx="18">
                   <c:v>13.000620371417984</c:v>
                 </c:pt>
-                <c:pt idx="14">
+                <c:pt idx="19">
                   <c:v>30.874999999999996</c:v>
                 </c:pt>
               </c:numCache>
@@ -1777,7 +1978,7 @@
             <c:multiLvlStrRef>
               <c:f>Building_MI!$A$6:$B$25</c:f>
               <c:multiLvlStrCache>
-                <c:ptCount val="15"/>
+                <c:ptCount val="20"/>
                 <c:lvl>
                   <c:pt idx="0">
                     <c:v>pre 1945</c:v>
@@ -1822,6 +2023,21 @@
                     <c:v>2000-2018</c:v>
                   </c:pt>
                   <c:pt idx="14">
+                    <c:v>2018-2050</c:v>
+                  </c:pt>
+                  <c:pt idx="15">
+                    <c:v>pre 1945</c:v>
+                  </c:pt>
+                  <c:pt idx="16">
+                    <c:v>1945-1970</c:v>
+                  </c:pt>
+                  <c:pt idx="17">
+                    <c:v>1970-2000</c:v>
+                  </c:pt>
+                  <c:pt idx="18">
+                    <c:v>2000-2018</c:v>
+                  </c:pt>
+                  <c:pt idx="19">
                     <c:v>2018-2050</c:v>
                   </c:pt>
                 </c:lvl>
@@ -1830,9 +2046,12 @@
                     <c:v>detached (vrijstaand)</c:v>
                   </c:pt>
                   <c:pt idx="5">
+                    <c:v>semi-detached (2-1 kap) / corner (hoek)</c:v>
+                  </c:pt>
+                  <c:pt idx="10">
                     <c:v>row house (tussenwoning)</c:v>
                   </c:pt>
-                  <c:pt idx="10">
+                  <c:pt idx="15">
                     <c:v>multiple fam (meergezins)</c:v>
                   </c:pt>
                 </c:lvl>
@@ -1861,33 +2080,48 @@
                   <c:v>11.134328358208954</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.22195400234333421</c:v>
+                  <c:v>0.18055071267605635</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>2.6977568010989645</c:v>
+                  <c:v>2.8769816441314555</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>4.4661873716387008</c:v>
+                  <c:v>4.8030037380281687</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>4.4661873716387008</c:v>
+                  <c:v>4.8030037380281687</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>8.1559276083351371</c:v>
+                  <c:v>11.134328358208954</c:v>
                 </c:pt>
                 <c:pt idx="10">
+                  <c:v>0.23043419420289715</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>2.6610480983091773</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>4.3972008869565204</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>4.3972008869565204</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>7.5458937198067639</c:v>
+                </c:pt>
+                <c:pt idx="15">
                   <c:v>0.23152289397233203</c:v>
                 </c:pt>
-                <c:pt idx="11">
+                <c:pt idx="16">
                   <c:v>2.9457613399785858</c:v>
                 </c:pt>
-                <c:pt idx="12">
+                <c:pt idx="17">
                   <c:v>4.8845030879199598</c:v>
                 </c:pt>
-                <c:pt idx="13">
+                <c:pt idx="18">
                   <c:v>4.8845030879199598</c:v>
                 </c:pt>
-                <c:pt idx="14">
+                <c:pt idx="19">
                   <c:v>5.8913043478260869</c:v>
                 </c:pt>
               </c:numCache>
@@ -1929,7 +2163,7 @@
             <c:multiLvlStrRef>
               <c:f>Building_MI!$A$6:$B$25</c:f>
               <c:multiLvlStrCache>
-                <c:ptCount val="15"/>
+                <c:ptCount val="20"/>
                 <c:lvl>
                   <c:pt idx="0">
                     <c:v>pre 1945</c:v>
@@ -1974,6 +2208,21 @@
                     <c:v>2000-2018</c:v>
                   </c:pt>
                   <c:pt idx="14">
+                    <c:v>2018-2050</c:v>
+                  </c:pt>
+                  <c:pt idx="15">
+                    <c:v>pre 1945</c:v>
+                  </c:pt>
+                  <c:pt idx="16">
+                    <c:v>1945-1970</c:v>
+                  </c:pt>
+                  <c:pt idx="17">
+                    <c:v>1970-2000</c:v>
+                  </c:pt>
+                  <c:pt idx="18">
+                    <c:v>2000-2018</c:v>
+                  </c:pt>
+                  <c:pt idx="19">
                     <c:v>2018-2050</c:v>
                   </c:pt>
                 </c:lvl>
@@ -1982,9 +2231,12 @@
                     <c:v>detached (vrijstaand)</c:v>
                   </c:pt>
                   <c:pt idx="5">
+                    <c:v>semi-detached (2-1 kap) / corner (hoek)</c:v>
+                  </c:pt>
+                  <c:pt idx="10">
                     <c:v>row house (tussenwoning)</c:v>
                   </c:pt>
-                  <c:pt idx="10">
+                  <c:pt idx="15">
                     <c:v>multiple fam (meergezins)</c:v>
                   </c:pt>
                 </c:lvl>
@@ -2013,33 +2265,48 @@
                   <c:v>34.328358208955223</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>68.748143953447638</c:v>
+                  <c:v>88.17859265915493</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>39.325271396191901</c:v>
+                  <c:v>48.554709943896711</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>23.837513570201232</c:v>
+                  <c:v>30.892644531220654</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>34.463428258368033</c:v>
+                  <c:v>42.414406792957749</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>26.505627658807413</c:v>
+                  <c:v>34.328358208955223</c:v>
                 </c:pt>
                 <c:pt idx="10">
+                  <c:v>64.768413495652169</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>37.434904464734288</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>22.392486746859905</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>32.834914582608697</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>24.90338164251208</c:v>
+                </c:pt>
+                <c:pt idx="15">
                   <c:v>33.943422969713424</c:v>
                 </c:pt>
-                <c:pt idx="11">
+                <c:pt idx="16">
                   <c:v>21.144124247640807</c:v>
                 </c:pt>
-                <c:pt idx="12">
+                <c:pt idx="17">
                   <c:v>12.026846123756583</c:v>
                 </c:pt>
-                <c:pt idx="13">
+                <c:pt idx="18">
                   <c:v>13.125159888908099</c:v>
                 </c:pt>
-                <c:pt idx="14">
+                <c:pt idx="19">
                   <c:v>2.206521739130435</c:v>
                 </c:pt>
               </c:numCache>
@@ -2078,7 +2345,7 @@
             <c:multiLvlStrRef>
               <c:f>Building_MI!$A$6:$B$25</c:f>
               <c:multiLvlStrCache>
-                <c:ptCount val="15"/>
+                <c:ptCount val="20"/>
                 <c:lvl>
                   <c:pt idx="0">
                     <c:v>pre 1945</c:v>
@@ -2123,6 +2390,21 @@
                     <c:v>2000-2018</c:v>
                   </c:pt>
                   <c:pt idx="14">
+                    <c:v>2018-2050</c:v>
+                  </c:pt>
+                  <c:pt idx="15">
+                    <c:v>pre 1945</c:v>
+                  </c:pt>
+                  <c:pt idx="16">
+                    <c:v>1945-1970</c:v>
+                  </c:pt>
+                  <c:pt idx="17">
+                    <c:v>1970-2000</c:v>
+                  </c:pt>
+                  <c:pt idx="18">
+                    <c:v>2000-2018</c:v>
+                  </c:pt>
+                  <c:pt idx="19">
                     <c:v>2018-2050</c:v>
                   </c:pt>
                 </c:lvl>
@@ -2131,9 +2413,12 @@
                     <c:v>detached (vrijstaand)</c:v>
                   </c:pt>
                   <c:pt idx="5">
+                    <c:v>semi-detached (2-1 kap) / corner (hoek)</c:v>
+                  </c:pt>
+                  <c:pt idx="10">
                     <c:v>row house (tussenwoning)</c:v>
                   </c:pt>
-                  <c:pt idx="10">
+                  <c:pt idx="15">
                     <c:v>multiple fam (meergezins)</c:v>
                   </c:pt>
                 </c:lvl>
@@ -2185,7 +2470,7 @@
             <c:multiLvlStrRef>
               <c:f>Building_MI!$A$6:$B$25</c:f>
               <c:multiLvlStrCache>
-                <c:ptCount val="15"/>
+                <c:ptCount val="20"/>
                 <c:lvl>
                   <c:pt idx="0">
                     <c:v>pre 1945</c:v>
@@ -2230,6 +2515,21 @@
                     <c:v>2000-2018</c:v>
                   </c:pt>
                   <c:pt idx="14">
+                    <c:v>2018-2050</c:v>
+                  </c:pt>
+                  <c:pt idx="15">
+                    <c:v>pre 1945</c:v>
+                  </c:pt>
+                  <c:pt idx="16">
+                    <c:v>1945-1970</c:v>
+                  </c:pt>
+                  <c:pt idx="17">
+                    <c:v>1970-2000</c:v>
+                  </c:pt>
+                  <c:pt idx="18">
+                    <c:v>2000-2018</c:v>
+                  </c:pt>
+                  <c:pt idx="19">
                     <c:v>2018-2050</c:v>
                   </c:pt>
                 </c:lvl>
@@ -2238,9 +2538,12 @@
                     <c:v>detached (vrijstaand)</c:v>
                   </c:pt>
                   <c:pt idx="5">
+                    <c:v>semi-detached (2-1 kap) / corner (hoek)</c:v>
+                  </c:pt>
+                  <c:pt idx="10">
                     <c:v>row house (tussenwoning)</c:v>
                   </c:pt>
-                  <c:pt idx="10">
+                  <c:pt idx="15">
                     <c:v>multiple fam (meergezins)</c:v>
                   </c:pt>
                 </c:lvl>
@@ -2269,33 +2572,48 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>274.30293953121662</c:v>
+                  <c:v>327.72170992957751</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>308.34079589176537</c:v>
+                  <c:v>394.5217951760564</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>478.53007769450903</c:v>
+                  <c:v>728.52222140845072</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>478.53007769450903</c:v>
+                  <c:v>728.52222140845072</c:v>
                 </c:pt>
                 <c:pt idx="9">
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="10">
+                  <c:v>263.36174559420294</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>290.68926591787442</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>427.32686753623187</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>427.32686753623187</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="15">
                   <c:v>224.76978087598758</c:v>
                 </c:pt>
-                <c:pt idx="11">
+                <c:pt idx="16">
                   <c:v>241.4403946610667</c:v>
                 </c:pt>
-                <c:pt idx="12">
+                <c:pt idx="17">
                   <c:v>324.79346358646245</c:v>
                 </c:pt>
-                <c:pt idx="13">
+                <c:pt idx="18">
                   <c:v>324.79346358646245</c:v>
                 </c:pt>
-                <c:pt idx="14">
+                <c:pt idx="19">
                   <c:v>0</c:v>
                 </c:pt>
               </c:numCache>
@@ -2337,7 +2655,7 @@
             <c:multiLvlStrRef>
               <c:f>Building_MI!$A$6:$B$25</c:f>
               <c:multiLvlStrCache>
-                <c:ptCount val="15"/>
+                <c:ptCount val="20"/>
                 <c:lvl>
                   <c:pt idx="0">
                     <c:v>pre 1945</c:v>
@@ -2382,6 +2700,21 @@
                     <c:v>2000-2018</c:v>
                   </c:pt>
                   <c:pt idx="14">
+                    <c:v>2018-2050</c:v>
+                  </c:pt>
+                  <c:pt idx="15">
+                    <c:v>pre 1945</c:v>
+                  </c:pt>
+                  <c:pt idx="16">
+                    <c:v>1945-1970</c:v>
+                  </c:pt>
+                  <c:pt idx="17">
+                    <c:v>1970-2000</c:v>
+                  </c:pt>
+                  <c:pt idx="18">
+                    <c:v>2000-2018</c:v>
+                  </c:pt>
+                  <c:pt idx="19">
                     <c:v>2018-2050</c:v>
                   </c:pt>
                 </c:lvl>
@@ -2390,9 +2723,12 @@
                     <c:v>detached (vrijstaand)</c:v>
                   </c:pt>
                   <c:pt idx="5">
+                    <c:v>semi-detached (2-1 kap) / corner (hoek)</c:v>
+                  </c:pt>
+                  <c:pt idx="10">
                     <c:v>row house (tussenwoning)</c:v>
                   </c:pt>
-                  <c:pt idx="10">
+                  <c:pt idx="15">
                     <c:v>multiple fam (meergezins)</c:v>
                   </c:pt>
                 </c:lvl>
@@ -2421,33 +2757,48 @@
                   <c:v>5.3582089552238799</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>2.8574045284956098</c:v>
+                  <c:v>3.3205046464788595</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>2.8574045284956098</c:v>
+                  <c:v>3.3205046464788595</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>2.8574045284956098</c:v>
+                  <c:v>3.3205046464788595</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>2.8574045284956098</c:v>
+                  <c:v>3.3205046464788595</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>6.3680452808421659</c:v>
+                  <c:v>5.3582089552238799</c:v>
                 </c:pt>
                 <c:pt idx="10">
+                  <c:v>2.7625526971014498</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>2.7625526971014502</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>2.7625526971014502</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>2.7625526971014498</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>6.57487922705314</c:v>
+                </c:pt>
+                <c:pt idx="15">
                   <c:v>12.270727132905126</c:v>
                 </c:pt>
-                <c:pt idx="11">
+                <c:pt idx="16">
                   <c:v>11.175228011281281</c:v>
                 </c:pt>
-                <c:pt idx="12">
+                <c:pt idx="17">
                   <c:v>5.6977324031620453</c:v>
                 </c:pt>
-                <c:pt idx="13">
+                <c:pt idx="18">
                   <c:v>5.6977324031620444</c:v>
                 </c:pt>
-                <c:pt idx="14">
+                <c:pt idx="19">
                   <c:v>12.581521739130434</c:v>
                 </c:pt>
               </c:numCache>
@@ -2489,7 +2840,7 @@
             <c:multiLvlStrRef>
               <c:f>Building_MI!$A$6:$B$25</c:f>
               <c:multiLvlStrCache>
-                <c:ptCount val="15"/>
+                <c:ptCount val="20"/>
                 <c:lvl>
                   <c:pt idx="0">
                     <c:v>pre 1945</c:v>
@@ -2534,6 +2885,21 @@
                     <c:v>2000-2018</c:v>
                   </c:pt>
                   <c:pt idx="14">
+                    <c:v>2018-2050</c:v>
+                  </c:pt>
+                  <c:pt idx="15">
+                    <c:v>pre 1945</c:v>
+                  </c:pt>
+                  <c:pt idx="16">
+                    <c:v>1945-1970</c:v>
+                  </c:pt>
+                  <c:pt idx="17">
+                    <c:v>1970-2000</c:v>
+                  </c:pt>
+                  <c:pt idx="18">
+                    <c:v>2000-2018</c:v>
+                  </c:pt>
+                  <c:pt idx="19">
                     <c:v>2018-2050</c:v>
                   </c:pt>
                 </c:lvl>
@@ -2542,9 +2908,12 @@
                     <c:v>detached (vrijstaand)</c:v>
                   </c:pt>
                   <c:pt idx="5">
+                    <c:v>semi-detached (2-1 kap) / corner (hoek)</c:v>
+                  </c:pt>
+                  <c:pt idx="10">
                     <c:v>row house (tussenwoning)</c:v>
                   </c:pt>
-                  <c:pt idx="10">
+                  <c:pt idx="15">
                     <c:v>multiple fam (meergezins)</c:v>
                   </c:pt>
                 </c:lvl>
@@ -2573,33 +2942,48 @@
                   <c:v>0.47761194029850745</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.43592320045376609</c:v>
+                  <c:v>0.84813828732394358</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0.43592320045376609</c:v>
+                  <c:v>0.84813828732394358</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0.43592320045376609</c:v>
+                  <c:v>0.84813828732394358</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>0.43592320045376609</c:v>
+                  <c:v>0.84813828732394358</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>0.56636311197635014</c:v>
+                  <c:v>0.47761194029850745</c:v>
                 </c:pt>
                 <c:pt idx="10">
+                  <c:v>0.35149360434782612</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>0.35149360434782612</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>0.35149360434782612</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>0.35149360434782612</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>0.58454106280193241</c:v>
+                </c:pt>
+                <c:pt idx="15">
                   <c:v>0.30749103120059285</c:v>
                 </c:pt>
-                <c:pt idx="11">
+                <c:pt idx="16">
                   <c:v>0.30764778053771408</c:v>
                 </c:pt>
-                <c:pt idx="12">
+                <c:pt idx="17">
                   <c:v>0.30850990193922923</c:v>
                 </c:pt>
-                <c:pt idx="13">
+                <c:pt idx="18">
                   <c:v>0.30890177551877468</c:v>
                 </c:pt>
-                <c:pt idx="14">
+                <c:pt idx="19">
                   <c:v>0.37499999999999994</c:v>
                 </c:pt>
               </c:numCache>
@@ -2642,7 +3026,7 @@
             <c:multiLvlStrRef>
               <c:f>Building_MI!$A$6:$B$25</c:f>
               <c:multiLvlStrCache>
-                <c:ptCount val="15"/>
+                <c:ptCount val="20"/>
                 <c:lvl>
                   <c:pt idx="0">
                     <c:v>pre 1945</c:v>
@@ -2687,6 +3071,21 @@
                     <c:v>2000-2018</c:v>
                   </c:pt>
                   <c:pt idx="14">
+                    <c:v>2018-2050</c:v>
+                  </c:pt>
+                  <c:pt idx="15">
+                    <c:v>pre 1945</c:v>
+                  </c:pt>
+                  <c:pt idx="16">
+                    <c:v>1945-1970</c:v>
+                  </c:pt>
+                  <c:pt idx="17">
+                    <c:v>1970-2000</c:v>
+                  </c:pt>
+                  <c:pt idx="18">
+                    <c:v>2000-2018</c:v>
+                  </c:pt>
+                  <c:pt idx="19">
                     <c:v>2018-2050</c:v>
                   </c:pt>
                 </c:lvl>
@@ -2695,9 +3094,12 @@
                     <c:v>detached (vrijstaand)</c:v>
                   </c:pt>
                   <c:pt idx="5">
+                    <c:v>semi-detached (2-1 kap) / corner (hoek)</c:v>
+                  </c:pt>
+                  <c:pt idx="10">
                     <c:v>row house (tussenwoning)</c:v>
                   </c:pt>
-                  <c:pt idx="10">
+                  <c:pt idx="15">
                     <c:v>multiple fam (meergezins)</c:v>
                   </c:pt>
                 </c:lvl>
@@ -2726,33 +3128,48 @@
                   <c:v>2.4029850746268657</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.88909868751549159</c:v>
+                  <c:v>1.2349096312676042</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>1.3217372921766131</c:v>
+                  <c:v>1.5919649113145524</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>1.8600312139951816</c:v>
+                  <c:v>1.8044713045070404</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>1.8600312139951813</c:v>
+                  <c:v>1.8044713045070404</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>2.7942562549570984</c:v>
+                  <c:v>2.4029850746268657</c:v>
                 </c:pt>
                 <c:pt idx="10">
+                  <c:v>0.81826993999999875</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>1.2663894665700473</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>1.8714109544927529</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>1.8714109544927526</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>2.8743961352657008</c:v>
+                </c:pt>
+                <c:pt idx="15">
                   <c:v>0.99483573656126456</c:v>
                 </c:pt>
-                <c:pt idx="11">
+                <c:pt idx="16">
                   <c:v>1.3383939973608361</c:v>
                 </c:pt>
-                <c:pt idx="12">
+                <c:pt idx="17">
                   <c:v>1.8858516190917312</c:v>
                 </c:pt>
-                <c:pt idx="13">
+                <c:pt idx="18">
                   <c:v>1.8877069491106706</c:v>
                 </c:pt>
-                <c:pt idx="14">
+                <c:pt idx="19">
                   <c:v>2.5054347826086953</c:v>
                 </c:pt>
               </c:numCache>
@@ -2795,7 +3212,7 @@
             <c:multiLvlStrRef>
               <c:f>Building_MI!$A$6:$B$25</c:f>
               <c:multiLvlStrCache>
-                <c:ptCount val="15"/>
+                <c:ptCount val="20"/>
                 <c:lvl>
                   <c:pt idx="0">
                     <c:v>pre 1945</c:v>
@@ -2840,6 +3257,21 @@
                     <c:v>2000-2018</c:v>
                   </c:pt>
                   <c:pt idx="14">
+                    <c:v>2018-2050</c:v>
+                  </c:pt>
+                  <c:pt idx="15">
+                    <c:v>pre 1945</c:v>
+                  </c:pt>
+                  <c:pt idx="16">
+                    <c:v>1945-1970</c:v>
+                  </c:pt>
+                  <c:pt idx="17">
+                    <c:v>1970-2000</c:v>
+                  </c:pt>
+                  <c:pt idx="18">
+                    <c:v>2000-2018</c:v>
+                  </c:pt>
+                  <c:pt idx="19">
                     <c:v>2018-2050</c:v>
                   </c:pt>
                 </c:lvl>
@@ -2848,9 +3280,12 @@
                     <c:v>detached (vrijstaand)</c:v>
                   </c:pt>
                   <c:pt idx="5">
+                    <c:v>semi-detached (2-1 kap) / corner (hoek)</c:v>
+                  </c:pt>
+                  <c:pt idx="10">
                     <c:v>row house (tussenwoning)</c:v>
                   </c:pt>
-                  <c:pt idx="10">
+                  <c:pt idx="15">
                     <c:v>multiple fam (meergezins)</c:v>
                   </c:pt>
                 </c:lvl>
@@ -2879,33 +3314,48 @@
                   <c:v>0.9253731343283581</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>1.4017232700569502</c:v>
+                  <c:v>1.6288591619718307</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>1.5076640921787434</c:v>
+                  <c:v>1.7222954333333333</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>1.5230046874033472</c:v>
+                  <c:v>1.7513309887323942</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>1.6046440721063466</c:v>
+                  <c:v>1.8392071225352109</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>0.81088831206287404</c:v>
+                  <c:v>0.9253731343283581</c:v>
                 </c:pt>
                 <c:pt idx="10">
+                  <c:v>1.3552014608695648</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>1.4637034560386468</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>1.4762390594202894</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>1.5566010376811577</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>0.7874396135265701</c:v>
+                </c:pt>
+                <c:pt idx="15">
                   <c:v>2.0525547885968374</c:v>
                 </c:pt>
-                <c:pt idx="11">
+                <c:pt idx="16">
                   <c:v>5.6162251376457508</c:v>
                 </c:pt>
-                <c:pt idx="12">
+                <c:pt idx="17">
                   <c:v>5.6058939766856062</c:v>
                 </c:pt>
-                <c:pt idx="13">
+                <c:pt idx="18">
                   <c:v>5.554137688621541</c:v>
                 </c:pt>
-                <c:pt idx="14">
+                <c:pt idx="19">
                   <c:v>0.99456521739130421</c:v>
                 </c:pt>
               </c:numCache>
@@ -2948,7 +3398,7 @@
             <c:multiLvlStrRef>
               <c:f>Building_MI!$A$6:$B$25</c:f>
               <c:multiLvlStrCache>
-                <c:ptCount val="15"/>
+                <c:ptCount val="20"/>
                 <c:lvl>
                   <c:pt idx="0">
                     <c:v>pre 1945</c:v>
@@ -2993,6 +3443,21 @@
                     <c:v>2000-2018</c:v>
                   </c:pt>
                   <c:pt idx="14">
+                    <c:v>2018-2050</c:v>
+                  </c:pt>
+                  <c:pt idx="15">
+                    <c:v>pre 1945</c:v>
+                  </c:pt>
+                  <c:pt idx="16">
+                    <c:v>1945-1970</c:v>
+                  </c:pt>
+                  <c:pt idx="17">
+                    <c:v>1970-2000</c:v>
+                  </c:pt>
+                  <c:pt idx="18">
+                    <c:v>2000-2018</c:v>
+                  </c:pt>
+                  <c:pt idx="19">
                     <c:v>2018-2050</c:v>
                   </c:pt>
                 </c:lvl>
@@ -3001,9 +3466,12 @@
                     <c:v>detached (vrijstaand)</c:v>
                   </c:pt>
                   <c:pt idx="5">
+                    <c:v>semi-detached (2-1 kap) / corner (hoek)</c:v>
+                  </c:pt>
+                  <c:pt idx="10">
                     <c:v>row house (tussenwoning)</c:v>
                   </c:pt>
-                  <c:pt idx="10">
+                  <c:pt idx="15">
                     <c:v>multiple fam (meergezins)</c:v>
                   </c:pt>
                 </c:lvl>
@@ -3025,20 +3493,14 @@
                 <c:pt idx="4">
                   <c:v>82.910447761194021</c:v>
                 </c:pt>
-                <c:pt idx="5">
-                  <c:v>0</c:v>
-                </c:pt>
                 <c:pt idx="6">
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="7">
                   <c:v>0</c:v>
                 </c:pt>
-                <c:pt idx="8">
-                  <c:v>0</c:v>
-                </c:pt>
                 <c:pt idx="9">
-                  <c:v>66.885983848871575</c:v>
+                  <c:v>82.910447761194021</c:v>
                 </c:pt>
                 <c:pt idx="11">
                   <c:v>0</c:v>
@@ -3047,6 +3509,15 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="14">
+                  <c:v>63.603864734299513</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="19">
                   <c:v>61.532608695652172</c:v>
                 </c:pt>
               </c:numCache>
@@ -3089,7 +3560,7 @@
             <c:multiLvlStrRef>
               <c:f>Building_MI!$A$6:$B$25</c:f>
               <c:multiLvlStrCache>
-                <c:ptCount val="15"/>
+                <c:ptCount val="20"/>
                 <c:lvl>
                   <c:pt idx="0">
                     <c:v>pre 1945</c:v>
@@ -3134,6 +3605,21 @@
                     <c:v>2000-2018</c:v>
                   </c:pt>
                   <c:pt idx="14">
+                    <c:v>2018-2050</c:v>
+                  </c:pt>
+                  <c:pt idx="15">
+                    <c:v>pre 1945</c:v>
+                  </c:pt>
+                  <c:pt idx="16">
+                    <c:v>1945-1970</c:v>
+                  </c:pt>
+                  <c:pt idx="17">
+                    <c:v>1970-2000</c:v>
+                  </c:pt>
+                  <c:pt idx="18">
+                    <c:v>2000-2018</c:v>
+                  </c:pt>
+                  <c:pt idx="19">
                     <c:v>2018-2050</c:v>
                   </c:pt>
                 </c:lvl>
@@ -3142,9 +3628,12 @@
                     <c:v>detached (vrijstaand)</c:v>
                   </c:pt>
                   <c:pt idx="5">
+                    <c:v>semi-detached (2-1 kap) / corner (hoek)</c:v>
+                  </c:pt>
+                  <c:pt idx="10">
                     <c:v>row house (tussenwoning)</c:v>
                   </c:pt>
-                  <c:pt idx="10">
+                  <c:pt idx="15">
                     <c:v>multiple fam (meergezins)</c:v>
                   </c:pt>
                 </c:lvl>
@@ -3166,18 +3655,12 @@
                 <c:pt idx="4">
                   <c:v>0</c:v>
                 </c:pt>
-                <c:pt idx="5">
-                  <c:v>0</c:v>
-                </c:pt>
                 <c:pt idx="6">
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="7">
                   <c:v>0</c:v>
                 </c:pt>
-                <c:pt idx="8">
-                  <c:v>0</c:v>
-                </c:pt>
                 <c:pt idx="9">
                   <c:v>0</c:v>
                 </c:pt>
@@ -3188,6 +3671,15 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="14">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="19">
                   <c:v>0</c:v>
                 </c:pt>
               </c:numCache>
@@ -3230,7 +3722,7 @@
             <c:multiLvlStrRef>
               <c:f>Building_MI!$A$6:$B$25</c:f>
               <c:multiLvlStrCache>
-                <c:ptCount val="15"/>
+                <c:ptCount val="20"/>
                 <c:lvl>
                   <c:pt idx="0">
                     <c:v>pre 1945</c:v>
@@ -3275,6 +3767,21 @@
                     <c:v>2000-2018</c:v>
                   </c:pt>
                   <c:pt idx="14">
+                    <c:v>2018-2050</c:v>
+                  </c:pt>
+                  <c:pt idx="15">
+                    <c:v>pre 1945</c:v>
+                  </c:pt>
+                  <c:pt idx="16">
+                    <c:v>1945-1970</c:v>
+                  </c:pt>
+                  <c:pt idx="17">
+                    <c:v>1970-2000</c:v>
+                  </c:pt>
+                  <c:pt idx="18">
+                    <c:v>2000-2018</c:v>
+                  </c:pt>
+                  <c:pt idx="19">
                     <c:v>2018-2050</c:v>
                   </c:pt>
                 </c:lvl>
@@ -3283,9 +3790,12 @@
                     <c:v>detached (vrijstaand)</c:v>
                   </c:pt>
                   <c:pt idx="5">
+                    <c:v>semi-detached (2-1 kap) / corner (hoek)</c:v>
+                  </c:pt>
+                  <c:pt idx="10">
                     <c:v>row house (tussenwoning)</c:v>
                   </c:pt>
-                  <c:pt idx="10">
+                  <c:pt idx="15">
                     <c:v>multiple fam (meergezins)</c:v>
                   </c:pt>
                 </c:lvl>
@@ -3314,33 +3824,48 @@
                   <c:v>0.11940298507462686</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>1.4468415957870977</c:v>
+                  <c:v>1.3351705873239421</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>1.4959366340908333</c:v>
+                  <c:v>1.3770228845070407</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>1.4959366340908333</c:v>
+                  <c:v>1.3770228845070407</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>1.4959366340908333</c:v>
+                  <c:v>1.3770228845070407</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>0.12054005335640638</c:v>
+                  <c:v>0.11940298507462686</c:v>
                 </c:pt>
                 <c:pt idx="10">
+                  <c:v>1.4697139710144911</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>1.5202924623188392</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>1.5202924623188392</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>1.5202924623188392</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>0.12077294685990339</c:v>
+                </c:pt>
+                <c:pt idx="15">
                   <c:v>0.72710811603260872</c:v>
                 </c:pt>
-                <c:pt idx="11">
+                <c:pt idx="16">
                   <c:v>0.74128453076004619</c:v>
                 </c:pt>
-                <c:pt idx="12">
+                <c:pt idx="17">
                   <c:v>0.74693622371541502</c:v>
                 </c:pt>
-                <c:pt idx="13">
+                <c:pt idx="18">
                   <c:v>0.74699402201086951</c:v>
                 </c:pt>
-                <c:pt idx="14">
+                <c:pt idx="19">
                   <c:v>0.12499999999999999</c:v>
                 </c:pt>
               </c:numCache>
@@ -3383,7 +3908,7 @@
             <c:multiLvlStrRef>
               <c:f>Building_MI!$A$6:$B$25</c:f>
               <c:multiLvlStrCache>
-                <c:ptCount val="15"/>
+                <c:ptCount val="20"/>
                 <c:lvl>
                   <c:pt idx="0">
                     <c:v>pre 1945</c:v>
@@ -3428,6 +3953,21 @@
                     <c:v>2000-2018</c:v>
                   </c:pt>
                   <c:pt idx="14">
+                    <c:v>2018-2050</c:v>
+                  </c:pt>
+                  <c:pt idx="15">
+                    <c:v>pre 1945</c:v>
+                  </c:pt>
+                  <c:pt idx="16">
+                    <c:v>1945-1970</c:v>
+                  </c:pt>
+                  <c:pt idx="17">
+                    <c:v>1970-2000</c:v>
+                  </c:pt>
+                  <c:pt idx="18">
+                    <c:v>2000-2018</c:v>
+                  </c:pt>
+                  <c:pt idx="19">
                     <c:v>2018-2050</c:v>
                   </c:pt>
                 </c:lvl>
@@ -3436,9 +3976,12 @@
                     <c:v>detached (vrijstaand)</c:v>
                   </c:pt>
                   <c:pt idx="5">
+                    <c:v>semi-detached (2-1 kap) / corner (hoek)</c:v>
+                  </c:pt>
+                  <c:pt idx="10">
                     <c:v>row house (tussenwoning)</c:v>
                   </c:pt>
-                  <c:pt idx="10">
+                  <c:pt idx="15">
                     <c:v>multiple fam (meergezins)</c:v>
                   </c:pt>
                 </c:lvl>
@@ -3470,30 +4013,45 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0.45927363478832417</c:v>
+                  <c:v>0.36854849295774644</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0.45927363478832417</c:v>
+                  <c:v>0.36854849295774644</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>0.45927363478832417</c:v>
+                  <c:v>0.36854849295774644</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>0.71860191794649941</c:v>
+                  <c:v>1.3731343283582089</c:v>
                 </c:pt>
                 <c:pt idx="10">
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="11">
+                  <c:v>0.47785589275362328</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>0.47785589275362328</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>0.47785589275362322</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>0.58454106280193241</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="16">
                   <c:v>0.35798067065217387</c:v>
                 </c:pt>
-                <c:pt idx="12">
+                <c:pt idx="17">
                   <c:v>0.35798067065217387</c:v>
                 </c:pt>
-                <c:pt idx="13">
+                <c:pt idx="18">
                   <c:v>0.35798067065217387</c:v>
                 </c:pt>
-                <c:pt idx="14">
+                <c:pt idx="19">
                   <c:v>0.27173913043478259</c:v>
                 </c:pt>
               </c:numCache>
@@ -3535,7 +4093,7 @@
             <c:multiLvlStrRef>
               <c:f>Building_MI!$A$6:$B$25</c:f>
               <c:multiLvlStrCache>
-                <c:ptCount val="15"/>
+                <c:ptCount val="20"/>
                 <c:lvl>
                   <c:pt idx="0">
                     <c:v>pre 1945</c:v>
@@ -3580,6 +4138,21 @@
                     <c:v>2000-2018</c:v>
                   </c:pt>
                   <c:pt idx="14">
+                    <c:v>2018-2050</c:v>
+                  </c:pt>
+                  <c:pt idx="15">
+                    <c:v>pre 1945</c:v>
+                  </c:pt>
+                  <c:pt idx="16">
+                    <c:v>1945-1970</c:v>
+                  </c:pt>
+                  <c:pt idx="17">
+                    <c:v>1970-2000</c:v>
+                  </c:pt>
+                  <c:pt idx="18">
+                    <c:v>2000-2018</c:v>
+                  </c:pt>
+                  <c:pt idx="19">
                     <c:v>2018-2050</c:v>
                   </c:pt>
                 </c:lvl>
@@ -3588,9 +4161,12 @@
                     <c:v>detached (vrijstaand)</c:v>
                   </c:pt>
                   <c:pt idx="5">
+                    <c:v>semi-detached (2-1 kap) / corner (hoek)</c:v>
+                  </c:pt>
+                  <c:pt idx="10">
                     <c:v>row house (tussenwoning)</c:v>
                   </c:pt>
-                  <c:pt idx="10">
+                  <c:pt idx="15">
                     <c:v>multiple fam (meergezins)</c:v>
                   </c:pt>
                 </c:lvl>
@@ -3619,33 +4195,48 @@
                   <c:v>25.686567164179102</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>52.610818815287224</c:v>
+                  <c:v>59.321162621126753</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>54.871576978276011</c:v>
+                  <c:v>61.770039730751165</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>56.267635468275145</c:v>
+                  <c:v>63.32280062112676</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>56.254998925480521</c:v>
+                  <c:v>63.308935043661968</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>29.146426562837981</c:v>
+                  <c:v>25.686567164179102</c:v>
                 </c:pt>
                 <c:pt idx="10">
+                  <c:v>51.236411047826117</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>53.458638824154598</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>54.822601641787458</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>54.810216828985524</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>29.855072463768114</c:v>
+                </c:pt>
+                <c:pt idx="15">
                   <c:v>69.102116075667027</c:v>
                 </c:pt>
-                <c:pt idx="11">
+                <c:pt idx="16">
                   <c:v>68.932509376387529</c:v>
                 </c:pt>
-                <c:pt idx="12">
+                <c:pt idx="17">
                   <c:v>70.660171043898245</c:v>
                 </c:pt>
-                <c:pt idx="13">
+                <c:pt idx="18">
                   <c:v>70.647256890612667</c:v>
                 </c:pt>
-                <c:pt idx="14">
+                <c:pt idx="19">
                   <c:v>21.673913043478258</c:v>
                 </c:pt>
               </c:numCache>
@@ -3687,7 +4278,7 @@
             <c:multiLvlStrRef>
               <c:f>Building_MI!$A$6:$B$25</c:f>
               <c:multiLvlStrCache>
-                <c:ptCount val="15"/>
+                <c:ptCount val="20"/>
                 <c:lvl>
                   <c:pt idx="0">
                     <c:v>pre 1945</c:v>
@@ -3732,6 +4323,21 @@
                     <c:v>2000-2018</c:v>
                   </c:pt>
                   <c:pt idx="14">
+                    <c:v>2018-2050</c:v>
+                  </c:pt>
+                  <c:pt idx="15">
+                    <c:v>pre 1945</c:v>
+                  </c:pt>
+                  <c:pt idx="16">
+                    <c:v>1945-1970</c:v>
+                  </c:pt>
+                  <c:pt idx="17">
+                    <c:v>1970-2000</c:v>
+                  </c:pt>
+                  <c:pt idx="18">
+                    <c:v>2000-2018</c:v>
+                  </c:pt>
+                  <c:pt idx="19">
                     <c:v>2018-2050</c:v>
                   </c:pt>
                 </c:lvl>
@@ -3740,9 +4346,12 @@
                     <c:v>detached (vrijstaand)</c:v>
                   </c:pt>
                   <c:pt idx="5">
+                    <c:v>semi-detached (2-1 kap) / corner (hoek)</c:v>
+                  </c:pt>
+                  <c:pt idx="10">
                     <c:v>row house (tussenwoning)</c:v>
                   </c:pt>
-                  <c:pt idx="10">
+                  <c:pt idx="15">
                     <c:v>multiple fam (meergezins)</c:v>
                   </c:pt>
                 </c:lvl>
@@ -3771,33 +4380,48 @@
                   <c:v>4.4776119402985072E-2</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.44418620022861793</c:v>
+                  <c:v>0.47078741830985782</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0.57625676755405841</c:v>
+                  <c:v>0.60906715422535074</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>1.2366096041812615</c:v>
+                  <c:v>1.3004658338028157</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>1.2366096041812615</c:v>
+                  <c:v>1.3004658338028157</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>8.7805177013483324E-2</c:v>
+                  <c:v>4.4776119402985072E-2</c:v>
                 </c:pt>
                 <c:pt idx="10">
+                  <c:v>0.43873775797101455</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>0.56953656787439622</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>1.2235306173913045</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>1.2235306173913045</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>9.6618357487922718E-2</c:v>
+                </c:pt>
+                <c:pt idx="15">
                   <c:v>0.83496118913043471</c:v>
                 </c:pt>
-                <c:pt idx="11">
+                <c:pt idx="16">
                   <c:v>0.7346677232625165</c:v>
                 </c:pt>
-                <c:pt idx="12">
+                <c:pt idx="17">
                   <c:v>0.88796920642292498</c:v>
                 </c:pt>
-                <c:pt idx="13">
+                <c:pt idx="18">
                   <c:v>0.88796920642292487</c:v>
                 </c:pt>
-                <c:pt idx="14">
+                <c:pt idx="19">
                   <c:v>0.53260869565217395</c:v>
                 </c:pt>
               </c:numCache>
@@ -3839,7 +4463,7 @@
             <c:multiLvlStrRef>
               <c:f>Building_MI!$A$6:$B$25</c:f>
               <c:multiLvlStrCache>
-                <c:ptCount val="15"/>
+                <c:ptCount val="20"/>
                 <c:lvl>
                   <c:pt idx="0">
                     <c:v>pre 1945</c:v>
@@ -3884,6 +4508,21 @@
                     <c:v>2000-2018</c:v>
                   </c:pt>
                   <c:pt idx="14">
+                    <c:v>2018-2050</c:v>
+                  </c:pt>
+                  <c:pt idx="15">
+                    <c:v>pre 1945</c:v>
+                  </c:pt>
+                  <c:pt idx="16">
+                    <c:v>1945-1970</c:v>
+                  </c:pt>
+                  <c:pt idx="17">
+                    <c:v>1970-2000</c:v>
+                  </c:pt>
+                  <c:pt idx="18">
+                    <c:v>2000-2018</c:v>
+                  </c:pt>
+                  <c:pt idx="19">
                     <c:v>2018-2050</c:v>
                   </c:pt>
                 </c:lvl>
@@ -3892,9 +4531,12 @@
                     <c:v>detached (vrijstaand)</c:v>
                   </c:pt>
                   <c:pt idx="5">
+                    <c:v>semi-detached (2-1 kap) / corner (hoek)</c:v>
+                  </c:pt>
+                  <c:pt idx="10">
                     <c:v>row house (tussenwoning)</c:v>
                   </c:pt>
-                  <c:pt idx="10">
+                  <c:pt idx="15">
                     <c:v>multiple fam (meergezins)</c:v>
                   </c:pt>
                 </c:lvl>
@@ -3923,33 +4565,48 @@
                   <c:v>99.507462686567166</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>24.733304291267608</c:v>
+                  <c:v>20.141574830985917</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>24.733304291267608</c:v>
+                  <c:v>20.141574830985917</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>24.733304291267608</c:v>
+                  <c:v>20.141574830985917</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>24.733304291267608</c:v>
+                  <c:v>20.141574830985917</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>123.76172759391449</c:v>
+                  <c:v>99.507462686567166</c:v>
                 </c:pt>
                 <c:pt idx="10">
+                  <c:v>25.673779000000003</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>25.673779000000003</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>25.673779000000003</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>25.673779000000003</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>128.72946859903382</c:v>
+                </c:pt>
+                <c:pt idx="15">
                   <c:v>16.468138358448616</c:v>
                 </c:pt>
-                <c:pt idx="11">
+                <c:pt idx="16">
                   <c:v>16.468138358448616</c:v>
                 </c:pt>
-                <c:pt idx="12">
+                <c:pt idx="17">
                   <c:v>16.468138358448616</c:v>
                 </c:pt>
-                <c:pt idx="13">
+                <c:pt idx="18">
                   <c:v>16.468138358448616</c:v>
                 </c:pt>
-                <c:pt idx="14">
+                <c:pt idx="19">
                   <c:v>30.114130434782606</c:v>
                 </c:pt>
               </c:numCache>
@@ -16293,7 +16950,7 @@
         <v>35.690020400000002</v>
       </c>
       <c r="K9" s="2">
-        <f t="shared" ref="K9:O10" si="1">$AG9*AI$35</f>
+        <f t="shared" ref="K9:O11" si="1">$AG9*AI$35</f>
         <v>0</v>
       </c>
       <c r="L9" s="2">
@@ -16434,110 +17091,86 @@
     </row>
     <row r="11" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A11" s="21" t="s">
-        <v>159</v>
+        <v>165</v>
       </c>
       <c r="B11" t="s">
         <v>164</v>
       </c>
       <c r="C11" s="2">
-        <f>0.17*Building_MI_periodharmonised!C11+0.83*Building_MI_periodharmonised!C16</f>
-        <v>0.3463036371951419</v>
+        <v>0.18886813098591554</v>
       </c>
       <c r="D11" s="2">
-        <f>0.17*Building_MI_periodharmonised!D11+0.83*Building_MI_periodharmonised!D16</f>
-        <v>189.94763395111249</v>
+        <v>322.16941545070426</v>
       </c>
       <c r="E11" s="2">
-        <f>0.17*Building_MI_periodharmonised!E11+0.83*Building_MI_periodharmonised!E16</f>
-        <v>1185.8494540952004</v>
+        <v>1388.6241446239421</v>
       </c>
       <c r="F11" s="2">
-        <f>0.17*Building_MI_periodharmonised!F11+0.83*Building_MI_periodharmonised!F16</f>
         <v>0</v>
       </c>
       <c r="G11" s="2">
-        <f>0.17*Building_MI_periodharmonised!G11+0.83*Building_MI_periodharmonised!G16</f>
-        <v>1.6904236620330679E-2</v>
+        <v>7.0422535211267607E-3</v>
       </c>
       <c r="H11" s="2">
-        <f>0.17*Building_MI_periodharmonised!H11+0.83*Building_MI_periodharmonised!H16</f>
-        <v>8.0895612976966706</v>
+        <v>10.021588338028154</v>
       </c>
       <c r="I11" s="2">
-        <f>0.17*Building_MI_periodharmonised!I11+0.83*Building_MI_periodharmonised!I16</f>
-        <v>0.22195400234333421</v>
+        <v>0.18055071267605635</v>
       </c>
       <c r="J11" s="2">
-        <f>0.17*Building_MI_periodharmonised!J11+0.83*Building_MI_periodharmonised!J16</f>
-        <v>68.748143953447638</v>
+        <v>88.17859265915493</v>
       </c>
       <c r="K11" s="2">
-        <f>0.17*Building_MI_periodharmonised!K11+0.83*Building_MI_periodharmonised!K16</f>
-        <v>4.9640352541771486</v>
+        <f t="shared" si="1"/>
+        <v>0</v>
       </c>
       <c r="L11" s="2">
-        <f>0.17*Building_MI_periodharmonised!L11+0.83*Building_MI_periodharmonised!L16</f>
-        <v>3.622404104399541</v>
+        <f t="shared" si="1"/>
+        <v>0</v>
       </c>
       <c r="M11" s="2">
-        <f>0.17*Building_MI_periodharmonised!M11+0.83*Building_MI_periodharmonised!M16</f>
-        <v>2.9515885295107371</v>
+        <f t="shared" si="1"/>
+        <v>0</v>
       </c>
       <c r="N11" s="2">
-        <f>0.17*Building_MI_periodharmonised!N11+0.83*Building_MI_periodharmonised!N16</f>
-        <v>1.0733049198220863</v>
+        <f t="shared" si="1"/>
+        <v>0</v>
       </c>
       <c r="O11" s="2">
-        <f>0.17*Building_MI_periodharmonised!O11+0.83*Building_MI_periodharmonised!O16</f>
-        <v>0.80497868986656462</v>
+        <f t="shared" si="1"/>
+        <v>0</v>
       </c>
       <c r="P11" s="2">
-        <f>0.17*Building_MI_periodharmonised!P11+0.83*Building_MI_periodharmonised!P16</f>
-        <v>274.30293953121662</v>
+        <v>327.72170992957751</v>
       </c>
       <c r="Q11" s="2">
-        <f>0.17*Building_MI_periodharmonised!Q11+0.83*Building_MI_periodharmonised!Q16</f>
-        <v>2.8574045284956098</v>
+        <v>3.3205046464788595</v>
       </c>
       <c r="R11" s="2">
-        <f>0.17*Building_MI_periodharmonised!R11+0.83*Building_MI_periodharmonised!R16</f>
-        <v>0.43592320045376609</v>
+        <v>0.84813828732394358</v>
       </c>
       <c r="S11" s="2">
-        <f>0.17*Building_MI_periodharmonised!S11+0.83*Building_MI_periodharmonised!S16</f>
-        <v>0.88909868751549159</v>
+        <v>1.2349096312676042</v>
       </c>
       <c r="T11" s="2">
-        <f>0.17*Building_MI_periodharmonised!T11+0.83*Building_MI_periodharmonised!T16</f>
-        <v>1.4017232700569502</v>
-      </c>
-      <c r="U11" s="2">
-        <f>0.17*Building_MI_periodharmonised!U11+0.83*Building_MI_periodharmonised!U16</f>
+        <v>1.6288591619718307</v>
+      </c>
+      <c r="U11" s="2"/>
+      <c r="V11" s="2"/>
+      <c r="W11" s="2">
+        <v>1.3351705873239421</v>
+      </c>
+      <c r="X11" s="2">
         <v>0</v>
       </c>
-      <c r="V11" s="2">
-        <f>0.17*Building_MI_periodharmonised!V11+0.83*Building_MI_periodharmonised!V16</f>
-        <v>0</v>
-      </c>
-      <c r="W11" s="2">
-        <f>0.17*Building_MI_periodharmonised!W11+0.83*Building_MI_periodharmonised!W16</f>
-        <v>1.4468415957870977</v>
-      </c>
-      <c r="X11" s="2">
-        <f>0.17*Building_MI_periodharmonised!X11+0.83*Building_MI_periodharmonised!X16</f>
-        <v>0</v>
-      </c>
       <c r="Y11" s="2">
-        <f>0.17*Building_MI_periodharmonised!Y11+0.83*Building_MI_periodharmonised!Y16</f>
-        <v>52.610818815287224</v>
+        <v>59.321162621126753</v>
       </c>
       <c r="Z11" s="2">
-        <f>0.17*Building_MI_periodharmonised!Z11+0.83*Building_MI_periodharmonised!Z16</f>
-        <v>0.44418620022861793</v>
+        <v>0.47078741830985782</v>
       </c>
       <c r="AA11" s="2">
-        <f>0.17*Building_MI_periodharmonised!AA11+0.83*Building_MI_periodharmonised!AA16</f>
-        <v>24.733304291267608</v>
+        <v>20.141574830985917</v>
       </c>
       <c r="AB11" s="2"/>
     </row>
@@ -16545,105 +17178,81 @@
       <c r="B12" t="s">
         <v>17</v>
       </c>
-      <c r="C12" s="2">
-        <f>0.17*Building_MI_periodharmonised!C12+0.83*Building_MI_periodharmonised!C17</f>
-        <v>0.42903842399299175</v>
+      <c r="C12" s="2" cm="1">
+        <f t="array" ref="C12:AA12">(25/30)*Building_MI_original_baseline!C12:AA12+(5/30)*Building_MI_original_baseline!C13:AA13</f>
+        <v>0.28178136220657279</v>
       </c>
       <c r="D12" s="2">
-        <f>0.17*Building_MI_periodharmonised!D12+0.83*Building_MI_periodharmonised!D17</f>
-        <v>170.95287055568011</v>
+        <v>289.95247390610336</v>
       </c>
       <c r="E12" s="2">
-        <f>0.17*Building_MI_periodharmonised!E12+0.83*Building_MI_periodharmonised!E17</f>
-        <v>1286.9143730009619</v>
+        <v>1521.8742804915478</v>
       </c>
       <c r="F12" s="2">
-        <f>0.17*Building_MI_periodharmonised!F12+0.83*Building_MI_periodharmonised!F17</f>
         <v>0</v>
       </c>
       <c r="G12" s="2">
-        <f>0.17*Building_MI_periodharmonised!G12+0.83*Building_MI_periodharmonised!G17</f>
-        <v>1.6904236620330679E-2</v>
+        <v>7.0422535211267616E-3</v>
       </c>
       <c r="H12" s="2">
-        <f>0.17*Building_MI_periodharmonised!H12+0.83*Building_MI_periodharmonised!H17</f>
-        <v>21.815203981267402</v>
+        <v>46.677546563380268</v>
       </c>
       <c r="I12" s="2">
-        <f>0.17*Building_MI_periodharmonised!I12+0.83*Building_MI_periodharmonised!I17</f>
-        <v>2.6977568010989645</v>
+        <v>2.8769816441314555</v>
       </c>
       <c r="J12" s="2">
-        <f>0.17*Building_MI_periodharmonised!J12+0.83*Building_MI_periodharmonised!J17</f>
-        <v>39.325271396191901</v>
+        <v>48.554709943896711</v>
       </c>
       <c r="K12" s="2">
-        <f>0.17*Building_MI_periodharmonised!K12+0.83*Building_MI_periodharmonised!K17</f>
-        <v>5.099357680378465</v>
+        <v>5.5396760193262908</v>
       </c>
       <c r="L12" s="2">
-        <f>0.17*Building_MI_periodharmonised!L12+0.83*Building_MI_periodharmonised!L17</f>
-        <v>3.7211529018977987</v>
+        <v>4.0424662843732397</v>
       </c>
       <c r="M12" s="2">
-        <f>0.17*Building_MI_periodharmonised!M12+0.83*Building_MI_periodharmonised!M17</f>
-        <v>3.0320505126574657</v>
+        <v>3.2938614168967133</v>
       </c>
       <c r="N12" s="2">
-        <f>0.17*Building_MI_periodharmonised!N12+0.83*Building_MI_periodharmonised!N17</f>
-        <v>1.1025638227845331</v>
+        <v>1.1977677879624411</v>
       </c>
       <c r="O12" s="2">
-        <f>0.17*Building_MI_periodharmonised!O12+0.83*Building_MI_periodharmonised!O17</f>
-        <v>0.82692286708839968</v>
+        <v>0.89832584097183088</v>
       </c>
       <c r="P12" s="2">
-        <f>0.17*Building_MI_periodharmonised!P12+0.83*Building_MI_periodharmonised!P17</f>
-        <v>308.34079589176537</v>
+        <v>394.5217951760564</v>
       </c>
       <c r="Q12" s="2">
-        <f>0.17*Building_MI_periodharmonised!Q12+0.83*Building_MI_periodharmonised!Q17</f>
-        <v>2.8574045284956098</v>
+        <v>3.3205046464788595</v>
       </c>
       <c r="R12" s="2">
-        <f>0.17*Building_MI_periodharmonised!R12+0.83*Building_MI_periodharmonised!R17</f>
-        <v>0.43592320045376609</v>
+        <v>0.84813828732394358</v>
       </c>
       <c r="S12" s="2">
-        <f>0.17*Building_MI_periodharmonised!S12+0.83*Building_MI_periodharmonised!S17</f>
-        <v>1.3217372921766131</v>
+        <v>1.5919649113145524</v>
       </c>
       <c r="T12" s="2">
-        <f>0.17*Building_MI_periodharmonised!T12+0.83*Building_MI_periodharmonised!T17</f>
-        <v>1.5076640921787434</v>
+        <v>1.7222954333333333</v>
       </c>
       <c r="U12" s="2">
-        <f>0.17*Building_MI_periodharmonised!U12+0.83*Building_MI_periodharmonised!U17</f>
         <v>0</v>
       </c>
       <c r="V12" s="2">
-        <f>0.17*Building_MI_periodharmonised!V12+0.83*Building_MI_periodharmonised!V17</f>
         <v>0</v>
       </c>
       <c r="W12" s="2">
-        <f>0.17*Building_MI_periodharmonised!W12+0.83*Building_MI_periodharmonised!W17</f>
-        <v>1.4959366340908333</v>
+        <v>1.3770228845070407</v>
       </c>
       <c r="X12" s="2">
-        <f>0.17*Building_MI_periodharmonised!X12+0.83*Building_MI_periodharmonised!X17</f>
-        <v>0.45927363478832417</v>
+        <v>0.36854849295774644</v>
       </c>
       <c r="Y12" s="2">
-        <f>0.17*Building_MI_periodharmonised!Y12+0.83*Building_MI_periodharmonised!Y17</f>
-        <v>54.871576978276011</v>
+        <v>61.770039730751165</v>
       </c>
       <c r="Z12" s="2">
-        <f>0.17*Building_MI_periodharmonised!Z12+0.83*Building_MI_periodharmonised!Z17</f>
-        <v>0.57625676755405841</v>
+        <v>0.60906715422535074</v>
       </c>
       <c r="AA12" s="2">
-        <f>0.17*Building_MI_periodharmonised!AA12+0.83*Building_MI_periodharmonised!AA17</f>
-        <v>24.733304291267608</v>
+        <v>20.141574830985917</v>
       </c>
       <c r="AB12" s="2"/>
     </row>
@@ -16651,105 +17260,81 @@
       <c r="B13" t="s">
         <v>18</v>
       </c>
-      <c r="C13" s="2">
-        <f>0.17*Building_MI_periodharmonised!C13+0.83*Building_MI_periodharmonised!C18</f>
-        <v>0.3567510263533375</v>
+      <c r="C13" s="2" cm="1">
+        <f t="array" ref="C13:AA13">(25/30)*Building_MI_original_baseline!C13:AA13+(5/30)*Building_MI_original_baseline!C14:AA14</f>
+        <v>0.25258702535211269</v>
       </c>
       <c r="D13" s="2">
-        <f>0.17*Building_MI_periodharmonised!D13+0.83*Building_MI_periodharmonised!D18</f>
-        <v>75.979053578518062</v>
+        <v>128.86776618309858</v>
       </c>
       <c r="E13" s="2">
-        <f>0.17*Building_MI_periodharmonised!E13+0.83*Building_MI_periodharmonised!E18</f>
-        <v>1353.0058488562827</v>
+        <v>1589.920186801407</v>
       </c>
       <c r="F13" s="2">
-        <f>0.17*Building_MI_periodharmonised!F13+0.83*Building_MI_periodharmonised!F18</f>
         <v>0</v>
       </c>
       <c r="G13" s="2">
-        <f>0.17*Building_MI_periodharmonised!G13+0.83*Building_MI_periodharmonised!G18</f>
-        <v>1.6904236620330679E-2</v>
+        <v>7.0422535211267616E-3</v>
       </c>
       <c r="H13" s="2">
-        <f>0.17*Building_MI_periodharmonised!H13+0.83*Building_MI_periodharmonised!H18</f>
-        <v>21.815203981267402</v>
+        <v>46.677546563380268</v>
       </c>
       <c r="I13" s="2">
-        <f>0.17*Building_MI_periodharmonised!I13+0.83*Building_MI_periodharmonised!I18</f>
-        <v>4.4661873716387008</v>
+        <v>4.8030037380281687</v>
       </c>
       <c r="J13" s="2">
-        <f>0.17*Building_MI_periodharmonised!J13+0.83*Building_MI_periodharmonised!J18</f>
-        <v>23.837513570201232</v>
+        <v>30.892644531220654</v>
       </c>
       <c r="K13" s="2">
-        <f>0.17*Building_MI_periodharmonised!K13+0.83*Building_MI_periodharmonised!K18</f>
-        <v>5.2944350486222076</v>
+        <v>5.7969504054659611</v>
       </c>
       <c r="L13" s="2">
-        <f>0.17*Building_MI_periodharmonised!L13+0.83*Building_MI_periodharmonised!L18</f>
-        <v>3.8635066571026933</v>
+        <v>4.2302070526373239</v>
       </c>
       <c r="M13" s="2">
-        <f>0.17*Building_MI_periodharmonised!M13+0.83*Building_MI_periodharmonised!M18</f>
-        <v>3.1480424613429352</v>
+        <v>3.446835376223004</v>
       </c>
       <c r="N13" s="2">
-        <f>0.17*Building_MI_periodharmonised!N13+0.83*Building_MI_periodharmonised!N18</f>
-        <v>1.1447427132156129</v>
+        <v>1.2533946822629107</v>
       </c>
       <c r="O13" s="2">
-        <f>0.17*Building_MI_periodharmonised!O13+0.83*Building_MI_periodharmonised!O18</f>
-        <v>0.85855703491170943</v>
+        <v>0.94004601169718272</v>
       </c>
       <c r="P13" s="2">
-        <f>0.17*Building_MI_periodharmonised!P13+0.83*Building_MI_periodharmonised!P18</f>
-        <v>478.53007769450903</v>
+        <v>728.52222140845072</v>
       </c>
       <c r="Q13" s="2">
-        <f>0.17*Building_MI_periodharmonised!Q13+0.83*Building_MI_periodharmonised!Q18</f>
-        <v>2.8574045284956098</v>
+        <v>3.3205046464788595</v>
       </c>
       <c r="R13" s="2">
-        <f>0.17*Building_MI_periodharmonised!R13+0.83*Building_MI_periodharmonised!R18</f>
-        <v>0.43592320045376609</v>
+        <v>0.84813828732394358</v>
       </c>
       <c r="S13" s="2">
-        <f>0.17*Building_MI_periodharmonised!S13+0.83*Building_MI_periodharmonised!S18</f>
-        <v>1.8600312139951816</v>
+        <v>1.8044713045070404</v>
       </c>
       <c r="T13" s="2">
-        <f>0.17*Building_MI_periodharmonised!T13+0.83*Building_MI_periodharmonised!T18</f>
-        <v>1.5230046874033472</v>
+        <v>1.7513309887323942</v>
       </c>
       <c r="U13" s="2">
-        <f>0.17*Building_MI_periodharmonised!U13+0.83*Building_MI_periodharmonised!U18</f>
         <v>0</v>
       </c>
       <c r="V13" s="2">
-        <f>0.17*Building_MI_periodharmonised!V13+0.83*Building_MI_periodharmonised!V18</f>
         <v>0</v>
       </c>
       <c r="W13" s="2">
-        <f>0.17*Building_MI_periodharmonised!W13+0.83*Building_MI_periodharmonised!W18</f>
-        <v>1.4959366340908333</v>
+        <v>1.3770228845070407</v>
       </c>
       <c r="X13" s="2">
-        <f>0.17*Building_MI_periodharmonised!X13+0.83*Building_MI_periodharmonised!X18</f>
-        <v>0.45927363478832417</v>
+        <v>0.36854849295774644</v>
       </c>
       <c r="Y13" s="2">
-        <f>0.17*Building_MI_periodharmonised!Y13+0.83*Building_MI_periodharmonised!Y18</f>
-        <v>56.267635468275145</v>
+        <v>63.32280062112676</v>
       </c>
       <c r="Z13" s="2">
-        <f>0.17*Building_MI_periodharmonised!Z13+0.83*Building_MI_periodharmonised!Z18</f>
-        <v>1.2366096041812615</v>
+        <v>1.3004658338028157</v>
       </c>
       <c r="AA13" s="2">
-        <f>0.17*Building_MI_periodharmonised!AA13+0.83*Building_MI_periodharmonised!AA18</f>
-        <v>24.733304291267608</v>
+        <v>20.141574830985917</v>
       </c>
       <c r="AB13" s="2"/>
     </row>
@@ -16758,104 +17343,80 @@
         <v>58</v>
       </c>
       <c r="C14" s="2">
-        <f>0.17*Building_MI_periodharmonised!C14+0.83*Building_MI_periodharmonised!C19</f>
-        <v>0.35675102635333744</v>
+        <v>0.25258702535211269</v>
       </c>
       <c r="D14" s="2">
-        <f>0.17*Building_MI_periodharmonised!D14+0.83*Building_MI_periodharmonised!D19</f>
-        <v>75.979053578518062</v>
+        <v>128.86776618309858</v>
       </c>
       <c r="E14" s="2">
-        <f>0.17*Building_MI_periodharmonised!E14+0.83*Building_MI_periodharmonised!E19</f>
-        <v>1353.0058488562825</v>
+        <v>1589.920186801407</v>
       </c>
       <c r="F14" s="2">
-        <f>0.17*Building_MI_periodharmonised!F14+0.83*Building_MI_periodharmonised!F19</f>
         <v>0</v>
       </c>
       <c r="G14" s="2">
-        <f>0.17*Building_MI_periodharmonised!G14+0.83*Building_MI_periodharmonised!G19</f>
-        <v>1.6904236620330679E-2</v>
+        <v>7.0422535211267607E-3</v>
       </c>
       <c r="H14" s="2">
-        <f>0.17*Building_MI_periodharmonised!H14+0.83*Building_MI_periodharmonised!H19</f>
-        <v>21.815203981267398</v>
+        <v>46.677546563380261</v>
       </c>
       <c r="I14" s="2">
-        <f>0.17*Building_MI_periodharmonised!I14+0.83*Building_MI_periodharmonised!I19</f>
-        <v>4.4661873716387008</v>
+        <v>4.8030037380281687</v>
       </c>
       <c r="J14" s="2">
-        <f>0.17*Building_MI_periodharmonised!J14+0.83*Building_MI_periodharmonised!J19</f>
-        <v>34.463428258368033</v>
+        <v>42.414406792957749</v>
       </c>
       <c r="K14" s="2">
-        <f>0.17*Building_MI_periodharmonised!K14+0.83*Building_MI_periodharmonised!K19</f>
-        <v>5.6673208462169828</v>
+        <f t="shared" ref="K14:O16" si="2">$AG14*AI$35</f>
+        <v>0</v>
       </c>
       <c r="L14" s="2">
-        <f>0.17*Building_MI_periodharmonised!L14+0.83*Building_MI_periodharmonised!L19</f>
-        <v>4.1356125094015841</v>
+        <f t="shared" si="2"/>
+        <v>0</v>
       </c>
       <c r="M14" s="2">
-        <f>0.17*Building_MI_periodharmonised!M14+0.83*Building_MI_periodharmonised!M19</f>
-        <v>3.3697583409938829</v>
+        <f t="shared" si="2"/>
+        <v>0</v>
       </c>
       <c r="N14" s="2">
-        <f>0.17*Building_MI_periodharmonised!N14+0.83*Building_MI_periodharmonised!N19</f>
-        <v>1.2253666694523211</v>
+        <f t="shared" si="2"/>
+        <v>0</v>
       </c>
       <c r="O14" s="2">
-        <f>0.17*Building_MI_periodharmonised!O14+0.83*Building_MI_periodharmonised!O19</f>
-        <v>0.91902500208924065</v>
+        <f t="shared" si="2"/>
+        <v>0</v>
       </c>
       <c r="P14" s="2">
-        <f>0.17*Building_MI_periodharmonised!P14+0.83*Building_MI_periodharmonised!P19</f>
-        <v>478.53007769450903</v>
+        <v>728.52222140845072</v>
       </c>
       <c r="Q14" s="2">
-        <f>0.17*Building_MI_periodharmonised!Q14+0.83*Building_MI_periodharmonised!Q19</f>
-        <v>2.8574045284956098</v>
+        <v>3.3205046464788595</v>
       </c>
       <c r="R14" s="2">
-        <f>0.17*Building_MI_periodharmonised!R14+0.83*Building_MI_periodharmonised!R19</f>
-        <v>0.43592320045376609</v>
+        <v>0.84813828732394358</v>
       </c>
       <c r="S14" s="2">
-        <f>0.17*Building_MI_periodharmonised!S14+0.83*Building_MI_periodharmonised!S19</f>
-        <v>1.8600312139951813</v>
+        <v>1.8044713045070404</v>
       </c>
       <c r="T14" s="2">
-        <f>0.17*Building_MI_periodharmonised!T14+0.83*Building_MI_periodharmonised!T19</f>
-        <v>1.6046440721063466</v>
-      </c>
-      <c r="U14" s="2">
-        <f>0.17*Building_MI_periodharmonised!U14+0.83*Building_MI_periodharmonised!U19</f>
-        <v>0</v>
-      </c>
-      <c r="V14" s="2">
-        <f>0.17*Building_MI_periodharmonised!V14+0.83*Building_MI_periodharmonised!V19</f>
-        <v>0</v>
-      </c>
+        <v>1.8392071225352109</v>
+      </c>
+      <c r="U14" s="2"/>
+      <c r="V14" s="2"/>
       <c r="W14" s="2">
-        <f>0.17*Building_MI_periodharmonised!W14+0.83*Building_MI_periodharmonised!W19</f>
-        <v>1.4959366340908333</v>
+        <v>1.3770228845070407</v>
       </c>
       <c r="X14" s="2">
-        <f>0.17*Building_MI_periodharmonised!X14+0.83*Building_MI_periodharmonised!X19</f>
-        <v>0.45927363478832417</v>
+        <v>0.36854849295774644</v>
       </c>
       <c r="Y14" s="2">
-        <f>0.17*Building_MI_periodharmonised!Y14+0.83*Building_MI_periodharmonised!Y19</f>
-        <v>56.254998925480521</v>
+        <v>63.308935043661968</v>
       </c>
       <c r="Z14" s="2">
-        <f>0.17*Building_MI_periodharmonised!Z14+0.83*Building_MI_periodharmonised!Z19</f>
-        <v>1.2366096041812615</v>
+        <v>1.3004658338028157</v>
       </c>
       <c r="AA14" s="2">
-        <f>0.17*Building_MI_periodharmonised!AA14+0.83*Building_MI_periodharmonised!AA19</f>
-        <v>24.733304291267608</v>
+        <v>20.141574830985917</v>
       </c>
       <c r="AB14" s="2"/>
     </row>
@@ -16864,250 +17425,230 @@
         <v>21</v>
       </c>
       <c r="C15" s="2">
-        <f>0.17*Building_MI_periodharmonised!C15+0.83*Building_MI_periodharmonised!C20</f>
-        <v>1.3014110606388347</v>
+        <v>1.8059701492537312</v>
       </c>
       <c r="D15" s="2">
-        <f>0.17*Building_MI_periodharmonised!D15+0.83*Building_MI_periodharmonised!D20</f>
-        <v>186.50297714326916</v>
+        <v>218.41791044776119</v>
       </c>
       <c r="E15" s="2">
-        <f>0.17*Building_MI_periodharmonised!E15+0.83*Building_MI_periodharmonised!E20</f>
-        <v>1582.3432165260654</v>
+        <v>1190.3880597014925</v>
       </c>
       <c r="F15" s="2">
-        <f>0.17*Building_MI_periodharmonised!F15+0.83*Building_MI_periodharmonised!F20</f>
-        <v>0.55104621818444022</v>
+        <v>0.10447761194029852</v>
       </c>
       <c r="G15" s="2">
-        <f>0.17*Building_MI_periodharmonised!G15+0.83*Building_MI_periodharmonised!G20</f>
-        <v>0.85236426562837997</v>
+        <v>0.62686567164179097</v>
       </c>
       <c r="H15" s="2">
-        <f>0.17*Building_MI_periodharmonised!H15+0.83*Building_MI_periodharmonised!H20</f>
-        <v>13.928634364409836</v>
+        <v>15.820895522388058</v>
       </c>
       <c r="I15" s="2">
-        <f>0.17*Building_MI_periodharmonised!I15+0.83*Building_MI_periodharmonised!I20</f>
-        <v>8.1559276083351371</v>
+        <v>11.134328358208954</v>
       </c>
       <c r="J15" s="2">
-        <f>0.17*Building_MI_periodharmonised!J15+0.83*Building_MI_periodharmonised!J20</f>
-        <v>26.505627658807413</v>
+        <v>34.328358208955223</v>
       </c>
       <c r="K15" s="2">
-        <f>0.17*Building_MI_periodharmonised!K15+0.83*Building_MI_periodharmonised!K20</f>
-        <v>10.257359081404573</v>
+        <f t="shared" si="2"/>
+        <v>0</v>
       </c>
       <c r="L15" s="2">
-        <f>0.17*Building_MI_periodharmonised!L15+0.83*Building_MI_periodharmonised!L20</f>
-        <v>7.4850998702141478</v>
+        <f t="shared" si="2"/>
+        <v>0</v>
       </c>
       <c r="M15" s="2">
-        <f>0.17*Building_MI_periodharmonised!M15+0.83*Building_MI_periodharmonised!M20</f>
-        <v>6.0989702646189352</v>
+        <f t="shared" si="2"/>
+        <v>0</v>
       </c>
       <c r="N15" s="2">
-        <f>0.17*Building_MI_periodharmonised!N15+0.83*Building_MI_periodharmonised!N20</f>
-        <v>2.2178073689523399</v>
+        <f t="shared" si="2"/>
+        <v>0</v>
       </c>
       <c r="O15" s="2">
-        <f>0.17*Building_MI_periodharmonised!O15+0.83*Building_MI_periodharmonised!O20</f>
-        <v>1.663355526714255</v>
+        <f t="shared" si="2"/>
+        <v>0</v>
       </c>
       <c r="P15" s="2">
-        <f>0.17*Building_MI_periodharmonised!P15+0.83*Building_MI_periodharmonised!P20</f>
         <v>0</v>
       </c>
       <c r="Q15" s="2">
-        <f>0.17*Building_MI_periodharmonised!Q15+0.83*Building_MI_periodharmonised!Q20</f>
-        <v>6.3680452808421659</v>
+        <v>5.3582089552238799</v>
       </c>
       <c r="R15" s="2">
-        <f>0.17*Building_MI_periodharmonised!R15+0.83*Building_MI_periodharmonised!R20</f>
-        <v>0.56636311197635014</v>
+        <v>0.47761194029850745</v>
       </c>
       <c r="S15" s="2">
-        <f>0.17*Building_MI_periodharmonised!S15+0.83*Building_MI_periodharmonised!S20</f>
-        <v>2.7942562549570984</v>
+        <v>2.4029850746268657</v>
       </c>
       <c r="T15" s="2">
-        <f>0.17*Building_MI_periodharmonised!T15+0.83*Building_MI_periodharmonised!T20</f>
-        <v>0.81088831206287404</v>
+        <v>0.9253731343283581</v>
       </c>
       <c r="U15" s="2">
-        <f>0.17*Building_MI_periodharmonised!U15+0.83*Building_MI_periodharmonised!U20</f>
-        <v>66.885983848871575</v>
+        <v>82.910447761194021</v>
       </c>
       <c r="V15" s="2">
-        <f>0.17*Building_MI_periodharmonised!V15+0.83*Building_MI_periodharmonised!V20</f>
         <v>0</v>
       </c>
       <c r="W15" s="2">
-        <f>0.17*Building_MI_periodharmonised!W15+0.83*Building_MI_periodharmonised!W20</f>
-        <v>0.12054005335640638</v>
+        <v>0.11940298507462686</v>
       </c>
       <c r="X15" s="2">
-        <f>0.17*Building_MI_periodharmonised!X15+0.83*Building_MI_periodharmonised!X20</f>
-        <v>0.71860191794649941</v>
+        <v>1.3731343283582089</v>
       </c>
       <c r="Y15" s="2">
-        <f>0.17*Building_MI_periodharmonised!Y15+0.83*Building_MI_periodharmonised!Y20</f>
-        <v>29.146426562837981</v>
+        <v>25.686567164179102</v>
       </c>
       <c r="Z15" s="2">
-        <f>0.17*Building_MI_periodharmonised!Z15+0.83*Building_MI_periodharmonised!Z20</f>
-        <v>8.7805177013483324E-2</v>
+        <v>4.4776119402985072E-2</v>
       </c>
       <c r="AA15" s="2">
-        <f>0.17*Building_MI_periodharmonised!AA15+0.83*Building_MI_periodharmonised!AA20</f>
-        <v>123.76172759391449</v>
+        <v>99.507462686567166</v>
       </c>
       <c r="AB15" s="2"/>
     </row>
     <row r="16" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A16" s="21" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="B16" t="s">
         <v>164</v>
       </c>
       <c r="C16" s="2">
-        <v>0.20221829725790513</v>
+        <v>0.37854946376811599</v>
       </c>
       <c r="D16" s="2">
-        <v>169.93780449011857</v>
+        <v>162.86606424637682</v>
       </c>
       <c r="E16" s="2">
-        <v>1421.6139480039028</v>
+        <v>1144.3172885652173</v>
       </c>
       <c r="F16" s="2">
         <v>0</v>
       </c>
       <c r="G16" s="2">
-        <v>3.2032279496047429E-2</v>
+        <v>1.8924160869565217E-2</v>
       </c>
       <c r="H16" s="2">
-        <v>13.986688577099798</v>
+        <v>7.6938449159420292</v>
       </c>
       <c r="I16" s="2">
-        <v>0.23152289397233203</v>
+        <v>0.23043419420289715</v>
       </c>
       <c r="J16" s="2">
-        <v>33.943422969713424</v>
+        <v>64.768413495652169</v>
       </c>
       <c r="K16" s="2">
-        <f>$AG16*AI$35</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="L16" s="2">
-        <f>$AG16*AJ$35</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="M16" s="2">
-        <f>$AG16*AK$35</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="N16" s="2">
-        <f>$AG16*AL$35</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="O16" s="2">
-        <f>$AG16*AM$35</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="P16" s="2">
-        <v>224.76978087598758</v>
+        <v>263.36174559420294</v>
       </c>
       <c r="Q16" s="2">
-        <v>12.270727132905126</v>
+        <v>2.7625526971014498</v>
       </c>
       <c r="R16" s="2">
-        <v>0.30749103120059285</v>
+        <v>0.35149360434782612</v>
       </c>
       <c r="S16" s="2">
-        <v>0.99483573656126456</v>
+        <v>0.81826993999999875</v>
       </c>
       <c r="T16" s="2">
-        <v>2.0525547885968374</v>
+        <v>1.3552014608695648</v>
       </c>
       <c r="U16" s="2"/>
       <c r="V16" s="2"/>
       <c r="W16" s="2">
-        <v>0.72710811603260872</v>
+        <v>1.4697139710144911</v>
       </c>
       <c r="X16" s="2">
         <v>0</v>
       </c>
       <c r="Y16" s="2">
-        <v>69.102116075667027</v>
+        <v>51.236411047826117</v>
       </c>
       <c r="Z16" s="2">
-        <v>0.83496118913043471</v>
+        <v>0.43873775797101455</v>
       </c>
       <c r="AA16" s="2">
-        <v>16.468138358448616</v>
+        <v>25.673779000000003</v>
       </c>
       <c r="AB16" s="2"/>
     </row>
-    <row r="17" spans="2:28" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:28" x14ac:dyDescent="0.2">
       <c r="B17" t="s">
         <v>17</v>
       </c>
       <c r="C17" s="2" cm="1">
-        <f t="array" ref="C17:AA17">(25/30)*Building_MI_original_baseline!C22:AA22+(5/30)*Building_MI_original_baseline!C23:AA23</f>
-        <v>0.30659409121376718</v>
+        <f t="array" ref="C17:AA17">(25/30)*Building_MI_original_baseline!C17:AA17+(5/30)*Building_MI_original_baseline!C18:AA18</f>
+        <v>0.45919950893719808</v>
       </c>
       <c r="D17" s="2">
-        <v>150.70739824798255</v>
+        <v>146.57945782125606</v>
       </c>
       <c r="E17" s="2">
-        <v>1514.6210843366187</v>
+        <v>1238.7900545992754</v>
       </c>
       <c r="F17" s="2">
-        <v>0.13764470016057295</v>
+        <v>0</v>
       </c>
       <c r="G17" s="2">
-        <v>3.2032279496047429E-2</v>
+        <v>1.8924160869565217E-2</v>
       </c>
       <c r="H17" s="2">
-        <v>13.822343876152829</v>
+        <v>16.722916946376813</v>
       </c>
       <c r="I17" s="2">
-        <v>2.9457613399785858</v>
+        <v>2.6610480983091773</v>
       </c>
       <c r="J17" s="2">
-        <v>21.144124247640807</v>
+        <v>37.434904464734288</v>
       </c>
       <c r="K17" s="2">
-        <v>6.7453931001493723</v>
+        <v>5.0091719964975852</v>
       </c>
       <c r="L17" s="2">
-        <v>4.9223138838927856</v>
+        <v>3.6553417271739135</v>
       </c>
       <c r="M17" s="2">
-        <v>4.0107742757644917</v>
+        <v>2.9784265925120779</v>
       </c>
       <c r="N17" s="2">
-        <v>1.4584633730052698</v>
+        <v>1.0830642154589376</v>
       </c>
       <c r="O17" s="2">
-        <v>1.0938475297539523</v>
+        <v>0.81229816159420298</v>
       </c>
       <c r="P17" s="2">
-        <v>241.4403946610667</v>
+        <v>290.68926591787442</v>
       </c>
       <c r="Q17" s="2">
-        <v>11.175228011281281</v>
+        <v>2.7625526971014502</v>
       </c>
       <c r="R17" s="2">
-        <v>0.30764778053771408</v>
+        <v>0.35149360434782612</v>
       </c>
       <c r="S17" s="2">
-        <v>1.3383939973608361</v>
+        <v>1.2663894665700473</v>
       </c>
       <c r="T17" s="2">
-        <v>5.6162251376457508</v>
+        <v>1.4637034560386468</v>
       </c>
       <c r="U17" s="2">
         <v>0</v>
@@ -17116,80 +17657,80 @@
         <v>0</v>
       </c>
       <c r="W17" s="2">
-        <v>0.74128453076004619</v>
+        <v>1.5202924623188392</v>
       </c>
       <c r="X17" s="2">
-        <v>0.35798067065217387</v>
+        <v>0.47785589275362328</v>
       </c>
       <c r="Y17" s="2">
-        <v>68.932509376387529</v>
+        <v>53.458638824154598</v>
       </c>
       <c r="Z17" s="2">
-        <v>0.7346677232625165</v>
+        <v>0.56953656787439622</v>
       </c>
       <c r="AA17" s="2">
-        <v>16.468138358448616</v>
+        <v>25.673779000000003</v>
       </c>
       <c r="AB17" s="2"/>
     </row>
-    <row r="18" spans="2:28" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:28" x14ac:dyDescent="0.2">
       <c r="B18" t="s">
         <v>18</v>
       </c>
       <c r="C18" s="2" cm="1">
-        <f t="array" ref="C18:AA18">(25/30)*Building_MI_original_baseline!C23:AA23+(5/30)*Building_MI_original_baseline!C24:AA24</f>
-        <v>0.78220971588438193</v>
+        <f t="array" ref="C18:AA18">(25/30)*Building_MI_original_baseline!C18:AA18+(5/30)*Building_MI_original_baseline!C19:AA19</f>
+        <v>0.37808582173913052</v>
       </c>
       <c r="D18" s="2">
-        <v>54.555367037302368</v>
+        <v>65.146425695652184</v>
       </c>
       <c r="E18" s="2">
-        <v>1526.4957120451579</v>
+        <v>1304.4812254217393</v>
       </c>
       <c r="F18" s="2">
-        <v>0.82586820096343772</v>
+        <v>0</v>
       </c>
       <c r="G18" s="2">
-        <v>3.2032279496047429E-2</v>
+        <v>1.8924160869565217E-2</v>
       </c>
       <c r="H18" s="2">
-        <v>13.000620371417984</v>
+        <v>16.722916946376813</v>
       </c>
       <c r="I18" s="2">
-        <v>4.8845030879199598</v>
+        <v>4.3972008869565204</v>
       </c>
       <c r="J18" s="2">
-        <v>12.026846123756583</v>
+        <v>22.392486746859905</v>
       </c>
       <c r="K18" s="2">
-        <v>4.835505887246395</v>
+        <v>5.1915102164975844</v>
       </c>
       <c r="L18" s="2">
-        <v>3.5286124042068292</v>
+        <v>3.7883993471739137</v>
       </c>
       <c r="M18" s="2">
-        <v>2.8751656626870461</v>
+        <v>3.0868439125120779</v>
       </c>
       <c r="N18" s="2">
-        <v>1.0455147864316532</v>
+        <v>1.1224886954589375</v>
       </c>
       <c r="O18" s="2">
-        <v>0.78413608982373983</v>
+        <v>0.84186652159420294</v>
       </c>
       <c r="P18" s="2">
-        <v>324.79346358646245</v>
+        <v>427.32686753623187</v>
       </c>
       <c r="Q18" s="2">
-        <v>5.6977324031620453</v>
+        <v>2.7625526971014502</v>
       </c>
       <c r="R18" s="2">
-        <v>0.30850990193922923</v>
+        <v>0.35149360434782612</v>
       </c>
       <c r="S18" s="2">
-        <v>1.8858516190917312</v>
+        <v>1.8714109544927529</v>
       </c>
       <c r="T18" s="2">
-        <v>5.6058939766856062</v>
+        <v>1.4762390594202894</v>
       </c>
       <c r="U18" s="2">
         <v>0</v>
@@ -17198,328 +17739,605 @@
         <v>0</v>
       </c>
       <c r="W18" s="2">
-        <v>0.74693622371541502</v>
+        <v>1.5202924623188392</v>
       </c>
       <c r="X18" s="2">
-        <v>0.35798067065217387</v>
+        <v>0.47785589275362328</v>
       </c>
       <c r="Y18" s="2">
-        <v>70.660171043898245</v>
+        <v>54.822601641787458</v>
       </c>
       <c r="Z18" s="2">
-        <v>0.88796920642292498</v>
+        <v>1.2235306173913045</v>
       </c>
       <c r="AA18" s="2">
-        <v>16.468138358448616</v>
+        <v>25.673779000000003</v>
       </c>
       <c r="AB18" s="2"/>
     </row>
-    <row r="19" spans="2:28" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:28" x14ac:dyDescent="0.2">
       <c r="B19" t="s">
         <v>58</v>
       </c>
       <c r="C19" s="2">
-        <v>0.78220971588438182</v>
+        <v>0.37808582173913047</v>
       </c>
       <c r="D19" s="2">
-        <v>54.555367037302368</v>
+        <v>65.146425695652184</v>
       </c>
       <c r="E19" s="2">
-        <v>1526.4957120451579</v>
+        <v>1304.4812254217391</v>
       </c>
       <c r="F19" s="2">
-        <v>0.82586820096343772</v>
+        <v>0</v>
       </c>
       <c r="G19" s="2">
-        <v>3.2032279496047429E-2</v>
+        <v>1.8924160869565217E-2</v>
       </c>
       <c r="H19" s="2">
-        <v>13.000620371417984</v>
+        <v>16.722916946376813</v>
       </c>
       <c r="I19" s="2">
-        <v>4.8845030879199598</v>
+        <v>4.3972008869565204</v>
       </c>
       <c r="J19" s="2">
-        <v>13.125159888908099</v>
+        <v>32.834914582608697</v>
       </c>
       <c r="K19" s="2">
-        <f t="shared" ref="K19:O20" si="2">$AG19*AI$35</f>
+        <f t="shared" ref="K19:O20" si="3">$AG19*AI$35</f>
         <v>0</v>
       </c>
       <c r="L19" s="2">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="M19" s="2">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="N19" s="2">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="O19" s="2">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="P19" s="2">
-        <v>324.79346358646245</v>
+        <v>427.32686753623187</v>
       </c>
       <c r="Q19" s="2">
-        <v>5.6977324031620444</v>
+        <v>2.7625526971014498</v>
       </c>
       <c r="R19" s="2">
-        <v>0.30890177551877468</v>
+        <v>0.35149360434782612</v>
       </c>
       <c r="S19" s="2">
-        <v>1.8877069491106706</v>
+        <v>1.8714109544927526</v>
       </c>
       <c r="T19" s="2">
-        <v>5.554137688621541</v>
+        <v>1.5566010376811577</v>
       </c>
       <c r="U19" s="2"/>
       <c r="V19" s="2"/>
       <c r="W19" s="2">
-        <v>0.74699402201086951</v>
+        <v>1.5202924623188392</v>
       </c>
       <c r="X19" s="2">
-        <v>0.35798067065217387</v>
+        <v>0.47785589275362322</v>
       </c>
       <c r="Y19" s="2">
-        <v>70.647256890612667</v>
+        <v>54.810216828985524</v>
       </c>
       <c r="Z19" s="2">
-        <v>0.88796920642292487</v>
+        <v>1.2235306173913045</v>
       </c>
       <c r="AA19" s="2">
-        <v>16.468138358448616</v>
+        <v>25.673779000000003</v>
       </c>
       <c r="AB19" s="2"/>
     </row>
-    <row r="20" spans="2:28" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:28" x14ac:dyDescent="0.2">
       <c r="B20" t="s">
         <v>21</v>
       </c>
       <c r="C20" s="2">
-        <v>1.5489130434782608</v>
+        <v>1.1980676328502415</v>
       </c>
       <c r="D20" s="2">
-        <v>237.06521739130437</v>
+        <v>179.96618357487924</v>
       </c>
       <c r="E20" s="2">
-        <v>1107.9076086956522</v>
+        <v>1662.6231884057972</v>
       </c>
       <c r="F20" s="2">
-        <v>0.31521739130434784</v>
+        <v>0.64251207729468607</v>
       </c>
       <c r="G20" s="2">
-        <v>1.2880434782608696</v>
+        <v>0.89855072463768126</v>
       </c>
       <c r="H20" s="2">
-        <v>30.874999999999996</v>
+        <v>13.54106280193237</v>
       </c>
       <c r="I20" s="2">
-        <v>5.8913043478260869</v>
+        <v>7.5458937198067639</v>
       </c>
       <c r="J20" s="2">
-        <v>2.206521739130435</v>
+        <v>24.90338164251208</v>
       </c>
       <c r="K20" s="2">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="L20" s="2">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="M20" s="2">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="N20" s="2">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="O20" s="2">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="P20" s="2">
         <v>0</v>
       </c>
       <c r="Q20" s="2">
-        <v>12.581521739130434</v>
+        <v>6.57487922705314</v>
       </c>
       <c r="R20" s="2">
-        <v>0.37499999999999994</v>
+        <v>0.58454106280193241</v>
       </c>
       <c r="S20" s="2">
-        <v>2.5054347826086953</v>
+        <v>2.8743961352657008</v>
       </c>
       <c r="T20" s="2">
-        <v>0.99456521739130421</v>
+        <v>0.7874396135265701</v>
       </c>
       <c r="U20" s="2">
-        <v>61.532608695652172</v>
+        <v>63.603864734299513</v>
       </c>
       <c r="V20" s="2">
         <v>0</v>
       </c>
       <c r="W20" s="2">
-        <v>0.12499999999999999</v>
+        <v>0.12077294685990339</v>
       </c>
       <c r="X20" s="2">
-        <v>0.27173913043478259</v>
+        <v>0.58454106280193241</v>
       </c>
       <c r="Y20" s="2">
-        <v>21.673913043478258</v>
+        <v>29.855072463768114</v>
       </c>
       <c r="Z20" s="2">
-        <v>0.53260869565217395</v>
+        <v>9.6618357487922718E-2</v>
       </c>
       <c r="AA20" s="2">
-        <v>30.114130434782606</v>
+        <v>128.72946859903382</v>
       </c>
       <c r="AB20" s="2"/>
     </row>
-    <row r="21" spans="2:28" x14ac:dyDescent="0.2">
-      <c r="C21" s="2"/>
-      <c r="D21" s="2"/>
-      <c r="E21" s="2"/>
-      <c r="F21" s="2"/>
-      <c r="G21" s="2"/>
-      <c r="H21" s="2"/>
-      <c r="I21" s="2"/>
-      <c r="J21" s="2"/>
-      <c r="K21" s="2"/>
-      <c r="L21" s="2"/>
-      <c r="M21" s="2"/>
-      <c r="N21" s="2"/>
-      <c r="O21" s="2"/>
-      <c r="P21" s="2"/>
-      <c r="Q21" s="2"/>
-      <c r="R21" s="2"/>
-      <c r="S21" s="2"/>
-      <c r="T21" s="2"/>
+    <row r="21" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="A21" s="21" t="s">
+        <v>161</v>
+      </c>
+      <c r="B21" t="s">
+        <v>164</v>
+      </c>
+      <c r="C21" s="2">
+        <v>0.20221829725790513</v>
+      </c>
+      <c r="D21" s="2">
+        <v>169.93780449011857</v>
+      </c>
+      <c r="E21" s="2">
+        <v>1421.6139480039028</v>
+      </c>
+      <c r="F21" s="2">
+        <v>0</v>
+      </c>
+      <c r="G21" s="2">
+        <v>3.2032279496047429E-2</v>
+      </c>
+      <c r="H21" s="2">
+        <v>13.986688577099798</v>
+      </c>
+      <c r="I21" s="2">
+        <v>0.23152289397233203</v>
+      </c>
+      <c r="J21" s="2">
+        <v>33.943422969713424</v>
+      </c>
+      <c r="K21" s="2">
+        <f>$AG21*AI$35</f>
+        <v>0</v>
+      </c>
+      <c r="L21" s="2">
+        <f>$AG21*AJ$35</f>
+        <v>0</v>
+      </c>
+      <c r="M21" s="2">
+        <f>$AG21*AK$35</f>
+        <v>0</v>
+      </c>
+      <c r="N21" s="2">
+        <f>$AG21*AL$35</f>
+        <v>0</v>
+      </c>
+      <c r="O21" s="2">
+        <f>$AG21*AM$35</f>
+        <v>0</v>
+      </c>
+      <c r="P21" s="2">
+        <v>224.76978087598758</v>
+      </c>
+      <c r="Q21" s="2">
+        <v>12.270727132905126</v>
+      </c>
+      <c r="R21" s="2">
+        <v>0.30749103120059285</v>
+      </c>
+      <c r="S21" s="2">
+        <v>0.99483573656126456</v>
+      </c>
+      <c r="T21" s="2">
+        <v>2.0525547885968374</v>
+      </c>
       <c r="U21" s="2"/>
       <c r="V21" s="2"/>
-      <c r="W21" s="2"/>
-      <c r="X21" s="2"/>
-      <c r="Y21" s="2"/>
-      <c r="Z21" s="2"/>
-      <c r="AA21" s="2"/>
+      <c r="W21" s="2">
+        <v>0.72710811603260872</v>
+      </c>
+      <c r="X21" s="2">
+        <v>0</v>
+      </c>
+      <c r="Y21" s="2">
+        <v>69.102116075667027</v>
+      </c>
+      <c r="Z21" s="2">
+        <v>0.83496118913043471</v>
+      </c>
+      <c r="AA21" s="2">
+        <v>16.468138358448616</v>
+      </c>
       <c r="AB21" s="2"/>
     </row>
-    <row r="22" spans="2:28" x14ac:dyDescent="0.2">
-      <c r="C22" s="2"/>
-      <c r="D22" s="2"/>
-      <c r="E22" s="2"/>
-      <c r="F22" s="2"/>
-      <c r="G22" s="2"/>
-      <c r="H22" s="2"/>
-      <c r="I22" s="2"/>
-      <c r="J22" s="2"/>
-      <c r="K22" s="2"/>
-      <c r="L22" s="2"/>
-      <c r="M22" s="2"/>
-      <c r="N22" s="2"/>
-      <c r="O22" s="2"/>
-      <c r="P22" s="2"/>
-      <c r="Q22" s="2"/>
-      <c r="R22" s="2"/>
-      <c r="S22" s="2"/>
-      <c r="T22" s="2"/>
-      <c r="U22" s="2"/>
-      <c r="V22" s="2"/>
-      <c r="W22" s="2"/>
-      <c r="X22" s="2"/>
-      <c r="Y22" s="2"/>
-      <c r="Z22" s="2"/>
-      <c r="AA22" s="2"/>
+    <row r="22" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="B22" t="s">
+        <v>17</v>
+      </c>
+      <c r="C22" s="2" cm="1">
+        <f t="array" ref="C22:AA22">(25/30)*Building_MI_original_baseline!C22:AA22+(5/30)*Building_MI_original_baseline!C23:AA23</f>
+        <v>0.30659409121376718</v>
+      </c>
+      <c r="D22" s="2">
+        <v>150.70739824798255</v>
+      </c>
+      <c r="E22" s="2">
+        <v>1514.6210843366187</v>
+      </c>
+      <c r="F22" s="2">
+        <v>0.13764470016057295</v>
+      </c>
+      <c r="G22" s="2">
+        <v>3.2032279496047429E-2</v>
+      </c>
+      <c r="H22" s="2">
+        <v>13.822343876152829</v>
+      </c>
+      <c r="I22" s="2">
+        <v>2.9457613399785858</v>
+      </c>
+      <c r="J22" s="2">
+        <v>21.144124247640807</v>
+      </c>
+      <c r="K22" s="2">
+        <v>6.7453931001493723</v>
+      </c>
+      <c r="L22" s="2">
+        <v>4.9223138838927856</v>
+      </c>
+      <c r="M22" s="2">
+        <v>4.0107742757644917</v>
+      </c>
+      <c r="N22" s="2">
+        <v>1.4584633730052698</v>
+      </c>
+      <c r="O22" s="2">
+        <v>1.0938475297539523</v>
+      </c>
+      <c r="P22" s="2">
+        <v>241.4403946610667</v>
+      </c>
+      <c r="Q22" s="2">
+        <v>11.175228011281281</v>
+      </c>
+      <c r="R22" s="2">
+        <v>0.30764778053771408</v>
+      </c>
+      <c r="S22" s="2">
+        <v>1.3383939973608361</v>
+      </c>
+      <c r="T22" s="2">
+        <v>5.6162251376457508</v>
+      </c>
+      <c r="U22" s="2">
+        <v>0</v>
+      </c>
+      <c r="V22" s="2">
+        <v>0</v>
+      </c>
+      <c r="W22" s="2">
+        <v>0.74128453076004619</v>
+      </c>
+      <c r="X22" s="2">
+        <v>0.35798067065217387</v>
+      </c>
+      <c r="Y22" s="2">
+        <v>68.932509376387529</v>
+      </c>
+      <c r="Z22" s="2">
+        <v>0.7346677232625165</v>
+      </c>
+      <c r="AA22" s="2">
+        <v>16.468138358448616</v>
+      </c>
       <c r="AB22" s="2"/>
     </row>
-    <row r="23" spans="2:28" x14ac:dyDescent="0.2">
-      <c r="C23" s="2"/>
-      <c r="D23" s="2"/>
-      <c r="E23" s="2"/>
-      <c r="F23" s="2"/>
-      <c r="G23" s="2"/>
-      <c r="H23" s="2"/>
-      <c r="I23" s="2"/>
-      <c r="J23" s="2"/>
-      <c r="K23" s="2"/>
-      <c r="L23" s="2"/>
-      <c r="M23" s="2"/>
-      <c r="N23" s="2"/>
-      <c r="O23" s="2"/>
-      <c r="P23" s="2"/>
-      <c r="Q23" s="2"/>
-      <c r="R23" s="2"/>
-      <c r="S23" s="2"/>
-      <c r="T23" s="2"/>
-      <c r="U23" s="2"/>
-      <c r="V23" s="2"/>
-      <c r="W23" s="2"/>
-      <c r="X23" s="2"/>
-      <c r="Y23" s="2"/>
-      <c r="Z23" s="2"/>
-      <c r="AA23" s="2"/>
+    <row r="23" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="B23" t="s">
+        <v>18</v>
+      </c>
+      <c r="C23" s="2" cm="1">
+        <f t="array" ref="C23:AA23">(25/30)*Building_MI_original_baseline!C23:AA23+(5/30)*Building_MI_original_baseline!C24:AA24</f>
+        <v>0.78220971588438193</v>
+      </c>
+      <c r="D23" s="2">
+        <v>54.555367037302368</v>
+      </c>
+      <c r="E23" s="2">
+        <v>1526.4957120451579</v>
+      </c>
+      <c r="F23" s="2">
+        <v>0.82586820096343772</v>
+      </c>
+      <c r="G23" s="2">
+        <v>3.2032279496047429E-2</v>
+      </c>
+      <c r="H23" s="2">
+        <v>13.000620371417984</v>
+      </c>
+      <c r="I23" s="2">
+        <v>4.8845030879199598</v>
+      </c>
+      <c r="J23" s="2">
+        <v>12.026846123756583</v>
+      </c>
+      <c r="K23" s="2">
+        <v>4.835505887246395</v>
+      </c>
+      <c r="L23" s="2">
+        <v>3.5286124042068292</v>
+      </c>
+      <c r="M23" s="2">
+        <v>2.8751656626870461</v>
+      </c>
+      <c r="N23" s="2">
+        <v>1.0455147864316532</v>
+      </c>
+      <c r="O23" s="2">
+        <v>0.78413608982373983</v>
+      </c>
+      <c r="P23" s="2">
+        <v>324.79346358646245</v>
+      </c>
+      <c r="Q23" s="2">
+        <v>5.6977324031620453</v>
+      </c>
+      <c r="R23" s="2">
+        <v>0.30850990193922923</v>
+      </c>
+      <c r="S23" s="2">
+        <v>1.8858516190917312</v>
+      </c>
+      <c r="T23" s="2">
+        <v>5.6058939766856062</v>
+      </c>
+      <c r="U23" s="2">
+        <v>0</v>
+      </c>
+      <c r="V23" s="2">
+        <v>0</v>
+      </c>
+      <c r="W23" s="2">
+        <v>0.74693622371541502</v>
+      </c>
+      <c r="X23" s="2">
+        <v>0.35798067065217387</v>
+      </c>
+      <c r="Y23" s="2">
+        <v>70.660171043898245</v>
+      </c>
+      <c r="Z23" s="2">
+        <v>0.88796920642292498</v>
+      </c>
+      <c r="AA23" s="2">
+        <v>16.468138358448616</v>
+      </c>
       <c r="AB23" s="2"/>
     </row>
-    <row r="24" spans="2:28" x14ac:dyDescent="0.2">
-      <c r="C24" s="2"/>
-      <c r="D24" s="2"/>
-      <c r="E24" s="2"/>
-      <c r="F24" s="2"/>
-      <c r="G24" s="2"/>
-      <c r="H24" s="2"/>
-      <c r="I24" s="2"/>
-      <c r="J24" s="2"/>
-      <c r="K24" s="2"/>
-      <c r="L24" s="2"/>
-      <c r="M24" s="2"/>
-      <c r="N24" s="2"/>
-      <c r="O24" s="2"/>
-      <c r="P24" s="2"/>
-      <c r="Q24" s="2"/>
-      <c r="R24" s="2"/>
-      <c r="S24" s="2"/>
-      <c r="T24" s="2"/>
+    <row r="24" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="B24" t="s">
+        <v>58</v>
+      </c>
+      <c r="C24" s="2">
+        <v>0.78220971588438182</v>
+      </c>
+      <c r="D24" s="2">
+        <v>54.555367037302368</v>
+      </c>
+      <c r="E24" s="2">
+        <v>1526.4957120451579</v>
+      </c>
+      <c r="F24" s="2">
+        <v>0.82586820096343772</v>
+      </c>
+      <c r="G24" s="2">
+        <v>3.2032279496047429E-2</v>
+      </c>
+      <c r="H24" s="2">
+        <v>13.000620371417984</v>
+      </c>
+      <c r="I24" s="2">
+        <v>4.8845030879199598</v>
+      </c>
+      <c r="J24" s="2">
+        <v>13.125159888908099</v>
+      </c>
+      <c r="K24" s="2">
+        <f>$AG24*AI$35</f>
+        <v>0</v>
+      </c>
+      <c r="L24" s="2">
+        <f>$AG24*AJ$35</f>
+        <v>0</v>
+      </c>
+      <c r="M24" s="2">
+        <f>$AG24*AK$35</f>
+        <v>0</v>
+      </c>
+      <c r="N24" s="2">
+        <f>$AG24*AL$35</f>
+        <v>0</v>
+      </c>
+      <c r="O24" s="2">
+        <f>$AG24*AM$35</f>
+        <v>0</v>
+      </c>
+      <c r="P24" s="2">
+        <v>324.79346358646245</v>
+      </c>
+      <c r="Q24" s="2">
+        <v>5.6977324031620444</v>
+      </c>
+      <c r="R24" s="2">
+        <v>0.30890177551877468</v>
+      </c>
+      <c r="S24" s="2">
+        <v>1.8877069491106706</v>
+      </c>
+      <c r="T24" s="2">
+        <v>5.554137688621541</v>
+      </c>
       <c r="U24" s="2"/>
       <c r="V24" s="2"/>
-      <c r="W24" s="2"/>
-      <c r="X24" s="2"/>
-      <c r="Y24" s="2"/>
-      <c r="Z24" s="2"/>
-      <c r="AA24" s="2"/>
+      <c r="W24" s="2">
+        <v>0.74699402201086951</v>
+      </c>
+      <c r="X24" s="2">
+        <v>0.35798067065217387</v>
+      </c>
+      <c r="Y24" s="2">
+        <v>70.647256890612667</v>
+      </c>
+      <c r="Z24" s="2">
+        <v>0.88796920642292487</v>
+      </c>
+      <c r="AA24" s="2">
+        <v>16.468138358448616</v>
+      </c>
       <c r="AB24" s="2"/>
     </row>
-    <row r="25" spans="2:28" x14ac:dyDescent="0.2">
-      <c r="C25" s="2"/>
-      <c r="D25" s="2"/>
-      <c r="E25" s="2"/>
-      <c r="F25" s="2"/>
-      <c r="G25" s="2"/>
-      <c r="H25" s="2"/>
-      <c r="I25" s="2"/>
-      <c r="J25" s="2"/>
-      <c r="K25" s="2"/>
-      <c r="L25" s="2"/>
-      <c r="M25" s="2"/>
-      <c r="N25" s="2"/>
-      <c r="O25" s="2"/>
-      <c r="P25" s="2"/>
-      <c r="Q25" s="2"/>
-      <c r="R25" s="2"/>
-      <c r="S25" s="2"/>
-      <c r="T25" s="2"/>
-      <c r="U25" s="2"/>
-      <c r="V25" s="2"/>
-      <c r="W25" s="2"/>
-      <c r="X25" s="2"/>
-      <c r="Y25" s="2"/>
-      <c r="Z25" s="2"/>
-      <c r="AA25" s="2"/>
+    <row r="25" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="B25" t="s">
+        <v>21</v>
+      </c>
+      <c r="C25" s="2">
+        <v>1.5489130434782608</v>
+      </c>
+      <c r="D25" s="2">
+        <v>237.06521739130437</v>
+      </c>
+      <c r="E25" s="2">
+        <v>1107.9076086956522</v>
+      </c>
+      <c r="F25" s="2">
+        <v>0.31521739130434784</v>
+      </c>
+      <c r="G25" s="2">
+        <v>1.2880434782608696</v>
+      </c>
+      <c r="H25" s="2">
+        <v>30.874999999999996</v>
+      </c>
+      <c r="I25" s="2">
+        <v>5.8913043478260869</v>
+      </c>
+      <c r="J25" s="2">
+        <v>2.206521739130435</v>
+      </c>
+      <c r="K25" s="2">
+        <f>$AG25*AI$35</f>
+        <v>0</v>
+      </c>
+      <c r="L25" s="2">
+        <f>$AG25*AJ$35</f>
+        <v>0</v>
+      </c>
+      <c r="M25" s="2">
+        <f>$AG25*AK$35</f>
+        <v>0</v>
+      </c>
+      <c r="N25" s="2">
+        <f>$AG25*AL$35</f>
+        <v>0</v>
+      </c>
+      <c r="O25" s="2">
+        <f>$AG25*AM$35</f>
+        <v>0</v>
+      </c>
+      <c r="P25" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q25" s="2">
+        <v>12.581521739130434</v>
+      </c>
+      <c r="R25" s="2">
+        <v>0.37499999999999994</v>
+      </c>
+      <c r="S25" s="2">
+        <v>2.5054347826086953</v>
+      </c>
+      <c r="T25" s="2">
+        <v>0.99456521739130421</v>
+      </c>
+      <c r="U25" s="2">
+        <v>61.532608695652172</v>
+      </c>
+      <c r="V25" s="2">
+        <v>0</v>
+      </c>
+      <c r="W25" s="2">
+        <v>0.12499999999999999</v>
+      </c>
+      <c r="X25" s="2">
+        <v>0.27173913043478259</v>
+      </c>
+      <c r="Y25" s="2">
+        <v>21.673913043478258</v>
+      </c>
+      <c r="Z25" s="2">
+        <v>0.53260869565217395</v>
+      </c>
+      <c r="AA25" s="2">
+        <v>30.114130434782606</v>
+      </c>
       <c r="AB25" s="2"/>
     </row>
     <row r="36" spans="1:33" x14ac:dyDescent="0.2">
@@ -17566,8 +18384,8 @@
   <mergeCells count="1">
     <mergeCell ref="AG36:AG38"/>
   </mergeCells>
-  <conditionalFormatting sqref="C6:C25 D11:AA15">
-    <cfRule type="colorScale" priority="135">
+  <conditionalFormatting sqref="C6:C10 C21:C25">
+    <cfRule type="colorScale" priority="187">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -17578,8 +18396,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D6:D10 D16:D25">
-    <cfRule type="colorScale" priority="138">
+  <conditionalFormatting sqref="AB6:AB10 AB21:AB25">
+    <cfRule type="colorScale" priority="262">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -17590,8 +18408,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E6:E10 E16:E25">
-    <cfRule type="colorScale" priority="141">
+  <conditionalFormatting sqref="AG6:AG10 AG16:AG25">
+    <cfRule type="colorScale" priority="265">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -17602,8 +18420,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F6:F10 F16:F25">
-    <cfRule type="colorScale" priority="144">
+  <conditionalFormatting sqref="D6:D10 D21:D25">
+    <cfRule type="colorScale" priority="269">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -17614,8 +18432,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G6:G10 G16:G25">
-    <cfRule type="colorScale" priority="147">
+  <conditionalFormatting sqref="E6:E10 E21:E25">
+    <cfRule type="colorScale" priority="271">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -17626,8 +18444,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H6:H10 H16:H25">
-    <cfRule type="colorScale" priority="150">
+  <conditionalFormatting sqref="F6:F10 F21:F25">
+    <cfRule type="colorScale" priority="273">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -17638,8 +18456,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I6:I10 I16:I25">
-    <cfRule type="colorScale" priority="153">
+  <conditionalFormatting sqref="G6:G10 G21:G25">
+    <cfRule type="colorScale" priority="275">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -17650,8 +18468,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J6:J10 J16:J25">
-    <cfRule type="colorScale" priority="156">
+  <conditionalFormatting sqref="H6:H10 H21:H25">
+    <cfRule type="colorScale" priority="277">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -17662,8 +18480,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K6:K10 K16:K25">
-    <cfRule type="colorScale" priority="159">
+  <conditionalFormatting sqref="I6:I10 I21:I25">
+    <cfRule type="colorScale" priority="279">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -17674,8 +18492,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L6:L10 L16:L25">
-    <cfRule type="colorScale" priority="162">
+  <conditionalFormatting sqref="J6:J10 J21:J25">
+    <cfRule type="colorScale" priority="281">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -17686,8 +18504,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="M6:M10 M16:M25">
-    <cfRule type="colorScale" priority="165">
+  <conditionalFormatting sqref="K6:K10 K21:K25">
+    <cfRule type="colorScale" priority="283">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -17698,8 +18516,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="N6:N10 N16:N25">
-    <cfRule type="colorScale" priority="168">
+  <conditionalFormatting sqref="L6:L10 L21:L25">
+    <cfRule type="colorScale" priority="285">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -17710,8 +18528,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="O6:O10 O16:O25">
-    <cfRule type="colorScale" priority="171">
+  <conditionalFormatting sqref="M6:M10 M21:M25">
+    <cfRule type="colorScale" priority="287">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -17722,8 +18540,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P6:P10 P16:P25">
-    <cfRule type="colorScale" priority="174">
+  <conditionalFormatting sqref="N6:N10 N21:N25">
+    <cfRule type="colorScale" priority="289">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -17734,8 +18552,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="Q6:Q10 Q16:Q25">
-    <cfRule type="colorScale" priority="177">
+  <conditionalFormatting sqref="O6:O10 O21:O25">
+    <cfRule type="colorScale" priority="291">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -17746,8 +18564,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="R6:R10 R16:R25">
-    <cfRule type="colorScale" priority="180">
+  <conditionalFormatting sqref="P6:P10 P21:P25">
+    <cfRule type="colorScale" priority="293">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -17758,8 +18576,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="S6:S10 S16:S25">
-    <cfRule type="colorScale" priority="183">
+  <conditionalFormatting sqref="Q6:Q10 Q21:Q25">
+    <cfRule type="colorScale" priority="295">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -17770,8 +18588,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="T6:T10 T16:T25">
-    <cfRule type="colorScale" priority="186">
+  <conditionalFormatting sqref="R6:R10 R21:R25">
+    <cfRule type="colorScale" priority="297">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -17782,8 +18600,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="U6:U10 U16:U25">
-    <cfRule type="colorScale" priority="189">
+  <conditionalFormatting sqref="S6:S10 S21:S25">
+    <cfRule type="colorScale" priority="299">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -17794,8 +18612,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="V6:V10 V16:V25">
-    <cfRule type="colorScale" priority="192">
+  <conditionalFormatting sqref="T6:T10 T21:T25">
+    <cfRule type="colorScale" priority="301">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -17806,8 +18624,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="W6:W10 W16:W25">
-    <cfRule type="colorScale" priority="195">
+  <conditionalFormatting sqref="U6:U10 U21:U25">
+    <cfRule type="colorScale" priority="303">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -17818,8 +18636,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="X6:X10 X16:X25">
-    <cfRule type="colorScale" priority="198">
+  <conditionalFormatting sqref="V6:V10 V21:V25">
+    <cfRule type="colorScale" priority="305">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -17830,8 +18648,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="Y6:Y10 Y16:Y25">
-    <cfRule type="colorScale" priority="201">
+  <conditionalFormatting sqref="W6:W10 W21:W25">
+    <cfRule type="colorScale" priority="307">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -17842,8 +18660,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="Z6:Z10 Z16:Z25">
-    <cfRule type="colorScale" priority="204">
+  <conditionalFormatting sqref="X6:X10 X21:X25">
+    <cfRule type="colorScale" priority="309">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -17854,8 +18672,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AA6:AA10 AA16:AA25">
-    <cfRule type="colorScale" priority="207">
+  <conditionalFormatting sqref="Y6:Y10 Y21:Y25">
+    <cfRule type="colorScale" priority="311">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -17866,8 +18684,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AB6:AB25">
-    <cfRule type="colorScale" priority="210">
+  <conditionalFormatting sqref="Z6:Z10 Z21:Z25">
+    <cfRule type="colorScale" priority="313">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -17878,8 +18696,632 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AG6:AG25">
-    <cfRule type="colorScale" priority="213">
+  <conditionalFormatting sqref="AA6:AA10 AA21:AA25">
+    <cfRule type="colorScale" priority="315">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C11:C15">
+    <cfRule type="colorScale" priority="52">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D11:D15">
+    <cfRule type="colorScale" priority="51">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E11:E15">
+    <cfRule type="colorScale" priority="50">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F11:F15">
+    <cfRule type="colorScale" priority="49">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G11:G15">
+    <cfRule type="colorScale" priority="48">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H11:H15">
+    <cfRule type="colorScale" priority="47">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I11:I15">
+    <cfRule type="colorScale" priority="46">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J11:J15">
+    <cfRule type="colorScale" priority="45">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K11:K15">
+    <cfRule type="colorScale" priority="44">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L11:L15">
+    <cfRule type="colorScale" priority="43">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="M11:M15">
+    <cfRule type="colorScale" priority="42">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="N11:N15">
+    <cfRule type="colorScale" priority="41">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="O11:O15">
+    <cfRule type="colorScale" priority="40">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="P11:P15">
+    <cfRule type="colorScale" priority="41">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="Q11:Q15">
+    <cfRule type="colorScale" priority="42">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="R11:R15">
+    <cfRule type="colorScale" priority="43">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="S11:S15">
+    <cfRule type="colorScale" priority="44">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="T11:T15">
+    <cfRule type="colorScale" priority="45">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="U11:U15">
+    <cfRule type="colorScale" priority="46">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="V11:V15">
+    <cfRule type="colorScale" priority="47">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="W11:W15">
+    <cfRule type="colorScale" priority="48">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="X11:X15">
+    <cfRule type="colorScale" priority="49">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="Y11:Y15">
+    <cfRule type="colorScale" priority="50">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="Z11:Z15">
+    <cfRule type="colorScale" priority="51">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AA11:AA15">
+    <cfRule type="colorScale" priority="52">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AB11:AB15">
+    <cfRule type="colorScale" priority="27">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C16:C20">
+    <cfRule type="colorScale" priority="7">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D16:D20">
+    <cfRule type="colorScale" priority="8">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E16:E20">
+    <cfRule type="colorScale" priority="9">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F16:F20">
+    <cfRule type="colorScale" priority="10">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G16:G20">
+    <cfRule type="colorScale" priority="11">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H16:H20">
+    <cfRule type="colorScale" priority="12">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I16:I20">
+    <cfRule type="colorScale" priority="13">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J16:J20">
+    <cfRule type="colorScale" priority="14">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K16:K20">
+    <cfRule type="colorScale" priority="6">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L16:L20">
+    <cfRule type="colorScale" priority="5">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="M16:M20">
+    <cfRule type="colorScale" priority="4">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="N16:N20">
+    <cfRule type="colorScale" priority="3">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="O16:O20">
+    <cfRule type="colorScale" priority="2">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="P16:P20">
+    <cfRule type="colorScale" priority="15">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="Q16:Q20">
+    <cfRule type="colorScale" priority="16">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="R16:R20">
+    <cfRule type="colorScale" priority="17">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="S16:S20">
+    <cfRule type="colorScale" priority="18">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="T16:T20">
+    <cfRule type="colorScale" priority="19">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="U16:U20">
+    <cfRule type="colorScale" priority="20">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="V16:V20">
+    <cfRule type="colorScale" priority="21">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="W16:W20">
+    <cfRule type="colorScale" priority="22">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="X16:X20">
+    <cfRule type="colorScale" priority="23">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="Y16:Y20">
+    <cfRule type="colorScale" priority="24">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="Z16:Z20">
+    <cfRule type="colorScale" priority="25">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AA16:AA20">
+    <cfRule type="colorScale" priority="26">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AB16:AB20">
+    <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>

</xml_diff>